<commit_message>
fix(export): ajustar estructura visual del Formulario 210 Excel para coincidir exactamente con el PDF oficial (10 columnas, layout fiel, paleta institucional)
</commit_message>
<xml_diff>
--- a/Formulario_210_2024_DIAN_Visual.xlsx
+++ b/Formulario_210_2024_DIAN_Visual.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="170" uniqueCount="170">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="169" uniqueCount="169">
   <si>
     <t>DIAN</t>
   </si>
@@ -74,7 +74,7 @@
       <rPr>
         <b/>
         <color rgb="FF000000"/>
-        <sz val="5.5"/>
+        <sz val="5"/>
         <rFont val="Arial"/>
       </rPr>
       <t xml:space="preserve">5. Número de Identificación Tributaria (NIT)
@@ -94,7 +94,7 @@
       <rPr>
         <b/>
         <color rgb="FF000000"/>
-        <sz val="5.5"/>
+        <sz val="5"/>
         <rFont val="Arial"/>
       </rPr>
       <t xml:space="preserve">6.DV
@@ -114,7 +114,7 @@
       <rPr>
         <b/>
         <color rgb="FF000000"/>
-        <sz val="5.5"/>
+        <sz val="5"/>
         <rFont val="Arial"/>
       </rPr>
       <t xml:space="preserve">7. Primer apellido
@@ -134,7 +134,7 @@
       <rPr>
         <b/>
         <color rgb="FF000000"/>
-        <sz val="5.5"/>
+        <sz val="5"/>
         <rFont val="Arial"/>
       </rPr>
       <t xml:space="preserve">8. Segundo apellido
@@ -154,7 +154,7 @@
       <rPr>
         <b/>
         <color rgb="FF000000"/>
-        <sz val="5.5"/>
+        <sz val="5"/>
         <rFont val="Arial"/>
       </rPr>
       <t xml:space="preserve">9. Primer nombre
@@ -174,7 +174,7 @@
       <rPr>
         <b/>
         <color rgb="FF000000"/>
-        <sz val="5.5"/>
+        <sz val="5"/>
         <rFont val="Arial"/>
       </rPr>
       <t xml:space="preserve">10. Otros nombres
@@ -194,7 +194,7 @@
       <rPr>
         <b/>
         <color rgb="FF000000"/>
-        <sz val="5.5"/>
+        <sz val="5"/>
         <rFont val="Arial"/>
       </rPr>
       <t xml:space="preserve">12.Cód. Dirección seccional
@@ -441,9 +441,6 @@
     <t>Liquidación privada del impuesto</t>
   </si>
   <si>
-    <t>Cédula general</t>
-  </si>
-  <si>
     <t>Ingresos brutos</t>
   </si>
   <si>
@@ -463,7 +460,7 @@
       <rPr>
         <b/>
         <color rgb="FF2E74B5"/>
-        <sz val="6"/>
+        <sz val="5.5"/>
         <rFont val="Arial"/>
       </rPr>
       <t xml:space="preserve">116 </t>
@@ -471,10 +468,10 @@
     <r>
       <rPr>
         <color rgb="FF444444"/>
-        <sz val="6"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">Impuesto s/ ren. líq. grav. cédula gral., pensiones y dividendos
+        <sz val="5.5"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">Impuesto s/ren.líq.grav. cédula gral., pensiones y dividendos
 </t>
     </r>
     <r>
@@ -497,7 +494,7 @@
       <rPr>
         <b/>
         <color rgb="FF2E74B5"/>
-        <sz val="6"/>
+        <sz val="5.5"/>
         <rFont val="Arial"/>
       </rPr>
       <t xml:space="preserve">117 </t>
@@ -505,7 +502,7 @@
     <r>
       <rPr>
         <color rgb="FF444444"/>
-        <sz val="6"/>
+        <sz val="5.5"/>
         <rFont val="Arial"/>
       </rPr>
       <t xml:space="preserve">Impuesto sobre renta presuntiva
@@ -540,7 +537,7 @@
       <rPr>
         <b/>
         <color rgb="FF2E74B5"/>
-        <sz val="6"/>
+        <sz val="5.5"/>
         <rFont val="Arial"/>
       </rPr>
       <t xml:space="preserve">118 </t>
@@ -548,10 +545,10 @@
     <r>
       <rPr>
         <color rgb="FF444444"/>
-        <sz val="6"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">Impuesto 2a. subcédula 2017 y sig. (art. 240 E.T.)
+        <sz val="5.5"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">Impuesto 2a. subcédula 2017 y sig. (art. 240)
 </t>
     </r>
     <r>
@@ -580,7 +577,7 @@
       <rPr>
         <b/>
         <color rgb="FF2E74B5"/>
-        <sz val="6"/>
+        <sz val="5.5"/>
         <rFont val="Arial"/>
       </rPr>
       <t xml:space="preserve">119 </t>
@@ -588,7 +585,7 @@
     <r>
       <rPr>
         <color rgb="FF444444"/>
-        <sz val="6"/>
+        <sz val="5.5"/>
         <rFont val="Arial"/>
       </rPr>
       <t xml:space="preserve">Impuesto dividendos 2016 y anteriores
@@ -623,7 +620,7 @@
       <rPr>
         <b/>
         <color rgb="FF2E74B5"/>
-        <sz val="6"/>
+        <sz val="5.5"/>
         <rFont val="Arial"/>
       </rPr>
       <t xml:space="preserve">120 </t>
@@ -631,10 +628,10 @@
     <r>
       <rPr>
         <color rgb="FF444444"/>
-        <sz val="6"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">Impuesto s/ dividendos y particip. del exterior
+        <sz val="5.5"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">Impuesto s/dividendos y particip. del exterior
 </t>
     </r>
     <r>
@@ -660,7 +657,7 @@
       <rPr>
         <b/>
         <color rgb="FF2E74B5"/>
-        <sz val="6"/>
+        <sz val="5.5"/>
         <rFont val="Arial"/>
       </rPr>
       <t xml:space="preserve">121 </t>
@@ -668,7 +665,7 @@
     <r>
       <rPr>
         <color rgb="FF444444"/>
-        <sz val="6"/>
+        <sz val="5.5"/>
         <rFont val="Arial"/>
       </rPr>
       <t xml:space="preserve">Total impuesto sobre rentas líquidas gravables
@@ -685,7 +682,8 @@
     </r>
   </si>
   <si>
-    <t>Aportes vol. AFC, FVP y AVC (art. 126-1 y 126-4)</t>
+    <t xml:space="preserve">Aportes vol. AFC, FVP y AVC
+(art. 126-1 y 126-4)</t>
   </si>
   <si>
     <t>35</t>
@@ -703,7 +701,8 @@
     <t>DESCUENTOS TRIBUTARIOS</t>
   </si>
   <si>
-    <t>Otras rentas exentas (incluye 25% num. 10 art. 206 E.T.)</t>
+    <t xml:space="preserve">Otras rentas exentas
+(incluye 25% num. 10 art. 206 E.T.)</t>
   </si>
   <si>
     <t>36</t>
@@ -722,7 +721,7 @@
       <rPr>
         <b/>
         <color rgb="FF2E74B5"/>
-        <sz val="6"/>
+        <sz val="5.5"/>
         <rFont val="Arial"/>
       </rPr>
       <t xml:space="preserve">122 </t>
@@ -730,10 +729,10 @@
     <r>
       <rPr>
         <color rgb="FF444444"/>
-        <sz val="6"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">Impuestos pagados en el exterior (arts. 254 y 255)
+        <sz val="5.5"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">Impuestos pagados en el exterior (arts.254 y 255)
 </t>
     </r>
     <r>
@@ -765,7 +764,7 @@
       <rPr>
         <b/>
         <color rgb="FF2E74B5"/>
-        <sz val="6"/>
+        <sz val="5.5"/>
         <rFont val="Arial"/>
       </rPr>
       <t xml:space="preserve">123 </t>
@@ -773,7 +772,7 @@
     <r>
       <rPr>
         <color rgb="FF444444"/>
-        <sz val="6"/>
+        <sz val="5.5"/>
         <rFont val="Arial"/>
       </rPr>
       <t xml:space="preserve">Donaciones (art. 257)
@@ -789,7 +788,8 @@
     </r>
   </si>
   <si>
-    <t>Intereses crédito de vivienda (art. 119 E.T.)</t>
+    <t xml:space="preserve">Intereses crédito de vivienda
+(art. 119 E.T.)</t>
   </si>
   <si>
     <t>38</t>
@@ -808,7 +808,7 @@
       <rPr>
         <b/>
         <color rgb="FF2E74B5"/>
-        <sz val="6"/>
+        <sz val="5.5"/>
         <rFont val="Arial"/>
       </rPr>
       <t xml:space="preserve">124 </t>
@@ -816,10 +816,10 @@
     <r>
       <rPr>
         <color rgb="FF444444"/>
-        <sz val="6"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">Dividendos, participaciones y otros (art. 258-1)
+        <sz val="5.5"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">Dividendos, participaciones y otros (art.258-1)
 </t>
     </r>
     <r>
@@ -833,7 +833,7 @@
   </si>
   <si>
     <t xml:space="preserve">Otras deducciones imputables
-(Dependientes, Salud, GMF, art. 387 E.T.)</t>
+(Dependientes, Salud, GMF, art. 387)</t>
   </si>
   <si>
     <t>39</t>
@@ -852,7 +852,7 @@
       <rPr>
         <b/>
         <color rgb="FF2E74B5"/>
-        <sz val="6"/>
+        <sz val="5.5"/>
         <rFont val="Arial"/>
       </rPr>
       <t xml:space="preserve">125 </t>
@@ -860,7 +860,7 @@
     <r>
       <rPr>
         <color rgb="FF444444"/>
-        <sz val="6"/>
+        <sz val="5.5"/>
         <rFont val="Arial"/>
       </rPr>
       <t xml:space="preserve">Total descuentos tributarios
@@ -896,7 +896,7 @@
       <rPr>
         <b/>
         <color rgb="FF2E74B5"/>
-        <sz val="6"/>
+        <sz val="5.5"/>
         <rFont val="Arial"/>
       </rPr>
       <t xml:space="preserve">126 </t>
@@ -904,7 +904,7 @@
     <r>
       <rPr>
         <color rgb="FF444444"/>
-        <sz val="6"/>
+        <sz val="5.5"/>
         <rFont val="Arial"/>
       </rPr>
       <t xml:space="preserve">Impuesto neto de renta
@@ -921,8 +921,8 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">Rentas exentas y/o deducciones imputables
-(limitadas 40%/1.340 UVT art. 336)</t>
+    <t xml:space="preserve">Rentas exentas y/o deduc. imputables
+(limit. 40%/1.340 UVT art. 336)</t>
   </si>
   <si>
     <t>41</t>
@@ -941,7 +941,7 @@
       <rPr>
         <b/>
         <color rgb="FF2E74B5"/>
-        <sz val="6"/>
+        <sz val="5.5"/>
         <rFont val="Arial"/>
       </rPr>
       <t xml:space="preserve">127 </t>
@@ -949,7 +949,7 @@
     <r>
       <rPr>
         <color rgb="FF444444"/>
-        <sz val="6"/>
+        <sz val="5.5"/>
         <rFont val="Arial"/>
       </rPr>
       <t xml:space="preserve">Impuesto de ganancias ocasionales
@@ -981,7 +981,7 @@
       <rPr>
         <b/>
         <color rgb="FF2E74B5"/>
-        <sz val="6"/>
+        <sz val="5.5"/>
         <rFont val="Arial"/>
       </rPr>
       <t xml:space="preserve">128 </t>
@@ -989,10 +989,10 @@
     <r>
       <rPr>
         <color rgb="FF444444"/>
-        <sz val="6"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">Desc. tributario por imp. pagados en el exterior por GO
+        <sz val="5.5"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">Desc. tributario por imp.pagados en el ext. por GO
 </t>
     </r>
     <r>
@@ -1021,7 +1021,7 @@
       <rPr>
         <b/>
         <color rgb="FF2E74B5"/>
-        <sz val="6"/>
+        <sz val="5.5"/>
         <rFont val="Arial"/>
       </rPr>
       <t xml:space="preserve">129 </t>
@@ -1029,7 +1029,7 @@
     <r>
       <rPr>
         <color rgb="FF444444"/>
-        <sz val="6"/>
+        <sz val="5.5"/>
         <rFont val="Arial"/>
       </rPr>
       <t xml:space="preserve">Total impuesto a cargo
@@ -1046,7 +1046,7 @@
     </r>
   </si>
   <si>
-    <t>Compensaciones por pérdidas de ejercicios anteriores</t>
+    <t>Compensaciones por pérdidas de ejerc. ant.</t>
   </si>
   <si>
     <t>56</t>
@@ -1062,7 +1062,7 @@
       <rPr>
         <b/>
         <color rgb="FF2E74B5"/>
-        <sz val="6"/>
+        <sz val="5.5"/>
         <rFont val="Arial"/>
       </rPr>
       <t xml:space="preserve">130 </t>
@@ -1070,10 +1070,10 @@
     <r>
       <rPr>
         <color rgb="FF444444"/>
-        <sz val="6"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">Anticipo renta liquidado año gravable anterior
+        <sz val="5.5"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">Anticipo renta liq. año gravable anterior (cas.133 dec.ant.)
 </t>
     </r>
     <r>
@@ -1105,7 +1105,7 @@
       <rPr>
         <b/>
         <color rgb="FF2E74B5"/>
-        <sz val="6"/>
+        <sz val="5.5"/>
         <rFont val="Arial"/>
       </rPr>
       <t xml:space="preserve">131 </t>
@@ -1113,10 +1113,10 @@
     <r>
       <rPr>
         <color rgb="FF444444"/>
-        <sz val="6"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">Saldo a favor año gravable anterior sin sol. de devolución
+        <sz val="5.5"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">Saldo a favor año grav. ant. sin sol. de devolución
 </t>
     </r>
     <r>
@@ -1133,7 +1133,7 @@
       <rPr>
         <b/>
         <color rgb="FF2E74B5"/>
-        <sz val="6"/>
+        <sz val="5.5"/>
         <rFont val="Arial"/>
       </rPr>
       <t xml:space="preserve">91 </t>
@@ -1144,7 +1144,7 @@
         <sz val="5.5"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">Ren. líq. cédula gral.
+      <t xml:space="preserve">Ren. líq. cédula general
 </t>
     </r>
     <r>
@@ -1161,7 +1161,7 @@
       <rPr>
         <b/>
         <color rgb="FF2E74B5"/>
-        <sz val="6"/>
+        <sz val="5.5"/>
         <rFont val="Arial"/>
       </rPr>
       <t xml:space="preserve">92 </t>
@@ -1189,7 +1189,7 @@
       <rPr>
         <b/>
         <color rgb="FF2E74B5"/>
-        <sz val="6"/>
+        <sz val="5.5"/>
         <rFont val="Arial"/>
       </rPr>
       <t xml:space="preserve">93 </t>
@@ -1218,7 +1218,7 @@
       <rPr>
         <b/>
         <color rgb="FF2E74B5"/>
-        <sz val="6"/>
+        <sz val="5.5"/>
         <rFont val="Arial"/>
       </rPr>
       <t xml:space="preserve">94 </t>
@@ -1246,7 +1246,7 @@
       <rPr>
         <b/>
         <color rgb="FF2E74B5"/>
-        <sz val="6"/>
+        <sz val="5.5"/>
         <rFont val="Arial"/>
       </rPr>
       <t xml:space="preserve">132 </t>
@@ -1274,7 +1274,7 @@
       <rPr>
         <b/>
         <color rgb="FF2E74B5"/>
-        <sz val="6"/>
+        <sz val="5.5"/>
         <rFont val="Arial"/>
       </rPr>
       <t xml:space="preserve">95 </t>
@@ -1285,7 +1285,7 @@
         <sz val="5.5"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">Comp. exc. ren. presuntiva
+      <t xml:space="preserve">Comp. exc. renta presuntiva
 </t>
     </r>
     <r>
@@ -1302,7 +1302,7 @@
       <rPr>
         <b/>
         <color rgb="FF2E74B5"/>
-        <sz val="6"/>
+        <sz val="5.5"/>
         <rFont val="Arial"/>
       </rPr>
       <t xml:space="preserve">96 </t>
@@ -1330,7 +1330,7 @@
       <rPr>
         <b/>
         <color rgb="FF2E74B5"/>
-        <sz val="6"/>
+        <sz val="5.5"/>
         <rFont val="Arial"/>
       </rPr>
       <t xml:space="preserve">97 </t>
@@ -1359,7 +1359,7 @@
       <rPr>
         <b/>
         <color rgb="FF2E74B5"/>
-        <sz val="6"/>
+        <sz val="5.5"/>
         <rFont val="Arial"/>
       </rPr>
       <t xml:space="preserve">98 </t>
@@ -1387,7 +1387,7 @@
       <rPr>
         <b/>
         <color rgb="FF2E74B5"/>
-        <sz val="6"/>
+        <sz val="5.5"/>
         <rFont val="Arial"/>
       </rPr>
       <t xml:space="preserve">133 </t>
@@ -1432,22 +1432,22 @@
         <sz val="6"/>
         <rFont val="Arial"/>
       </rPr>
-      <t>Ingresos brutos de pensiones de jubilación, invalidez, vejez, de sobrevivientes y riesgos profesionales del país y del exterior</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FF2E74B5"/>
-        <sz val="6"/>
+      <t>Ingresos brutos de pensiones del país y del exterior</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FF2E74B5"/>
+        <sz val="5.5"/>
         <rFont val="Arial"/>
       </rPr>
       <t xml:space="preserve">134 </t>
     </r>
     <r>
       <rPr>
-        <color rgb="FF000000"/>
+        <color rgb="FF444444"/>
         <sz val="5.5"/>
         <rFont val="Arial"/>
       </rPr>
@@ -1487,14 +1487,14 @@
       <rPr>
         <b/>
         <color rgb="FF2E74B5"/>
-        <sz val="6"/>
+        <sz val="5.5"/>
         <rFont val="Arial"/>
       </rPr>
       <t xml:space="preserve">135 </t>
     </r>
     <r>
       <rPr>
-        <color rgb="FF000000"/>
+        <color rgb="FF444444"/>
         <sz val="5.5"/>
         <rFont val="Arial"/>
       </rPr>
@@ -1546,7 +1546,7 @@
         <sz val="6"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">Total saldo a pagar
+      <t xml:space="preserve">TOTAL SALDO A PAGAR
 </t>
     </r>
     <r>
@@ -1575,7 +1575,7 @@
         <sz val="6"/>
         <rFont val="Arial"/>
       </rPr>
-      <t>Rentas exentas de pensiones (art. 206-1 E.T.)</t>
+      <t>Rentas exentas de pensiones (art. 206-1)</t>
     </r>
   </si>
   <si>
@@ -1595,7 +1595,7 @@
         <sz val="6"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">Total saldo a favor
+      <t xml:space="preserve">TOTAL SALDO A FAVOR
 </t>
     </r>
     <r>
@@ -1632,14 +1632,14 @@
       <rPr>
         <b/>
         <color rgb="FF2E74B5"/>
-        <sz val="6"/>
+        <sz val="5.5"/>
         <rFont val="Arial"/>
       </rPr>
       <t xml:space="preserve">138 </t>
     </r>
     <r>
       <rPr>
-        <color rgb="FF000000"/>
+        <color rgb="FF444444"/>
         <sz val="5.5"/>
         <rFont val="Arial"/>
       </rPr>
@@ -1663,18 +1663,18 @@
       <rPr>
         <b/>
         <color rgb="FF2E74B5"/>
-        <sz val="6"/>
+        <sz val="5.5"/>
         <rFont val="Arial"/>
       </rPr>
       <t xml:space="preserve">139 </t>
     </r>
     <r>
       <rPr>
-        <color rgb="FF000000"/>
-        <sz val="5.5"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">Adición al límite de deducciones (cas. 92 art. 336 inc. 2)
+        <color rgb="FF444444"/>
+        <sz val="5.5"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">Adición al límite de deducciones (cas. 92)
 </t>
     </r>
     <r>
@@ -1710,14 +1710,14 @@
       <rPr>
         <b/>
         <color rgb="FF2E74B5"/>
-        <sz val="6"/>
+        <sz val="5.5"/>
         <rFont val="Arial"/>
       </rPr>
       <t xml:space="preserve">140 </t>
     </r>
     <r>
       <rPr>
-        <color rgb="FF000000"/>
+        <color rgb="FF444444"/>
         <sz val="5.5"/>
         <rFont val="Arial"/>
       </rPr>
@@ -1757,14 +1757,14 @@
       <rPr>
         <b/>
         <color rgb="FF2E74B5"/>
-        <sz val="6"/>
+        <sz val="5.5"/>
         <rFont val="Arial"/>
       </rPr>
       <t xml:space="preserve">141 </t>
     </r>
     <r>
       <rPr>
-        <color rgb="FF000000"/>
+        <color rgb="FF444444"/>
         <sz val="5.5"/>
         <rFont val="Arial"/>
       </rPr>
@@ -1818,7 +1818,7 @@
         <sz val="6"/>
         <rFont val="Arial"/>
       </rPr>
-      <t>Subcédula 2017 y siguientes Numeral 3 art. 49 del E.T.</t>
+      <t>Subcédula 2017 y siguientes num. 3 art. 49</t>
     </r>
   </si>
   <si>
@@ -1867,26 +1867,26 @@
         <sz val="6"/>
         <rFont val="Arial"/>
       </rPr>
-      <t>Subcédula 2017 y siguientes Parágrafo 2 art. 49 del E.T.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FF2E74B5"/>
-        <sz val="6"/>
+      <t>Subcédula 2017 y siguientes par. 2 art. 49</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FF2E74B5"/>
+        <sz val="5.5"/>
         <rFont val="Arial"/>
       </rPr>
       <t xml:space="preserve">981 </t>
     </r>
     <r>
       <rPr>
-        <color rgb="FF000000"/>
-        <sz val="5.5"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">Cód. Representación / Firma del Declarante o de quien lo representa
+        <color rgb="FF444444"/>
+        <sz val="5.5"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">Cód. Rep./Firma del Declarante
 </t>
     </r>
     <r>
@@ -1914,26 +1914,26 @@
         <sz val="6"/>
         <rFont val="Arial"/>
       </rPr>
-      <t>Dividendos y participaciones recibidas del exterior</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FF2E74B5"/>
-        <sz val="6"/>
+      <t>Dividendos y participaciones del exterior</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FF2E74B5"/>
+        <sz val="5.5"/>
         <rFont val="Arial"/>
       </rPr>
       <t xml:space="preserve">982 </t>
     </r>
     <r>
       <rPr>
-        <color rgb="FF000000"/>
-        <sz val="5.5"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">Firma Contador Público / 994. Con salvedades
+        <color rgb="FF444444"/>
+        <sz val="5.5"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">Firma Contador / 994. Con salvedades
 </t>
     </r>
     <r>
@@ -1969,14 +1969,14 @@
       <rPr>
         <b/>
         <color rgb="FF2E74B5"/>
-        <sz val="6"/>
+        <sz val="5.5"/>
         <rFont val="Arial"/>
       </rPr>
       <t xml:space="preserve">983 </t>
     </r>
     <r>
       <rPr>
-        <color rgb="FF000000"/>
+        <color rgb="FF444444"/>
         <sz val="5.5"/>
         <rFont val="Arial"/>
       </rPr>
@@ -2008,26 +2008,26 @@
         <sz val="6"/>
         <rFont val="Arial"/>
       </rPr>
-      <t>Renta líquida gravable (Cédula gral.o ren. presuntiva, de pensiones y de dividendos y particip. del exterior)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FF2E74B5"/>
-        <sz val="6"/>
+      <t>Renta líq. grav. dividendos (base art. 241)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FF2E74B5"/>
+        <sz val="5.5"/>
         <rFont val="Arial"/>
       </rPr>
       <t xml:space="preserve">997 </t>
     </r>
     <r>
       <rPr>
-        <color rgb="FF000000"/>
-        <sz val="5.5"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">Espacio exclusivo para el sello de la entidad recaudadora
+        <color rgb="FF444444"/>
+        <sz val="5.5"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">Sello entidad recaudadora
 </t>
     </r>
     <r>
@@ -2047,18 +2047,18 @@
       <rPr>
         <b/>
         <color rgb="FF2E74B5"/>
-        <sz val="6"/>
+        <sz val="5.5"/>
         <rFont val="Arial"/>
       </rPr>
       <t xml:space="preserve">996 </t>
     </r>
     <r>
       <rPr>
-        <color rgb="FF000000"/>
-        <sz val="5.5"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">No. para el número interno de la DIAN / Adhesivo
+        <color rgb="FF444444"/>
+        <sz val="5.5"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">No. interno DIAN / Adhesivo
 </t>
     </r>
     <r>
@@ -2086,7 +2086,7 @@
         <sz val="6"/>
         <rFont val="Arial"/>
       </rPr>
-      <t>Ingresos por ganancias ocasionales del país y del exterior</t>
+      <t>Ingresos por ganancias ocasionales</t>
     </r>
   </si>
   <si>
@@ -2178,7 +2178,7 @@
       <name val="Arial Black"/>
     </font>
     <font>
-      <color rgb="FF2D6187"/>
+      <color rgb="FF2E74B5"/>
       <sz val="7"/>
       <name val="Arial"/>
     </font>
@@ -2197,29 +2197,29 @@
     <font>
       <b/>
       <color rgb="FF000000"/>
+      <sz val="6"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <color rgb="FF000000"/>
       <sz val="6.5"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
-      <color rgb="FFFFFFFF"/>
-      <sz val="7"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <color rgb="FF000000"/>
-      <sz val="7"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <b/>
       <color rgb="FF2E74B5"/>
-      <sz val="6.5"/>
+      <sz val="6"/>
       <name val="Arial"/>
     </font>
     <font>
       <color rgb="FF000000"/>
       <sz val="8"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FF000000"/>
+      <sz val="6.5"/>
       <name val="Arial"/>
     </font>
     <font>
@@ -2287,7 +2287,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="24">
+  <borders count="22">
     <border>
       <left/>
       <right/>
@@ -2512,40 +2512,10 @@
       <right style="medium">
         <color rgb="FF000000"/>
       </right>
-      <top style="thin">
+      <top style="medium">
         <color rgb="FF000000"/>
       </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="thick">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
+      <bottom style="medium">
         <color rgb="FF000000"/>
       </bottom>
       <diagonal/>
@@ -2554,6 +2524,21 @@
       <left style="thin">
         <color rgb="FF000000"/>
       </left>
+      <right style="thick">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thick">
+        <color rgb="FF000000"/>
+      </left>
       <right style="thin">
         <color rgb="FF000000"/>
       </right>
@@ -2569,7 +2554,7 @@
       <left style="thin">
         <color rgb="FF000000"/>
       </left>
-      <right style="thick">
+      <right style="thin">
         <color rgb="FF000000"/>
       </right>
       <top style="thin">
@@ -2596,21 +2581,6 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thick">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left style="thin">
         <color rgb="FF000000"/>
       </left>
@@ -2644,7 +2614,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="56">
+  <cellXfs count="52">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -2679,6 +2649,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -2688,11 +2659,11 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="14" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="12" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="5" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2704,95 +2675,82 @@
     <xf numFmtId="0" fontId="6" fillId="6" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="3" fontId="11" fillId="2" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="10" fillId="2" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="7" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="18" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="7" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="3" fontId="11" fillId="7" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="10" fillId="7" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="3" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="19" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="3" fontId="11" fillId="3" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="10" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="3" fontId="11" fillId="5" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="20" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="20" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="20" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="20" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="20" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="13" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="11" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="22" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="22" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="3" fontId="12" fillId="9" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="22" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="20" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3135,92 +3093,82 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L49"/>
+  <dimension ref="A1:J49"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="3.2" customWidth="1"/>
-    <col min="2" max="2" width="25" customWidth="1"/>
-    <col min="3" max="3" width="4.2" customWidth="1"/>
-    <col min="4" max="4" width="12.5" customWidth="1"/>
-    <col min="5" max="5" width="4.2" customWidth="1"/>
-    <col min="6" max="6" width="12.5" customWidth="1"/>
-    <col min="7" max="7" width="4.2" customWidth="1"/>
-    <col min="8" max="8" width="12.5" customWidth="1"/>
-    <col min="9" max="9" width="4.2" customWidth="1"/>
-    <col min="10" max="10" width="12.5" customWidth="1"/>
-    <col min="11" max="11" width="4.2" customWidth="1"/>
-    <col min="12" max="12" width="18" customWidth="1"/>
+    <col min="1" max="1" width="25" customWidth="1"/>
+    <col min="2" max="2" width="4.5" customWidth="1"/>
+    <col min="3" max="3" width="13" customWidth="1"/>
+    <col min="4" max="4" width="4.5" customWidth="1"/>
+    <col min="5" max="5" width="13" customWidth="1"/>
+    <col min="6" max="6" width="4.5" customWidth="1"/>
+    <col min="7" max="7" width="13" customWidth="1"/>
+    <col min="8" max="8" width="4.5" customWidth="1"/>
+    <col min="9" max="9" width="13" customWidth="1"/>
+    <col min="10" max="10" width="23" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="13" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="1" ht="14" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="2" t="s">
+      <c r="C1" s="2" t="s">
         <v>1</v>
       </c>
+      <c r="D1" s="2"/>
       <c r="E1" s="2"/>
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
-      <c r="H1" s="2"/>
-      <c r="I1" s="2"/>
-      <c r="J1" s="3"/>
-      <c r="K1" s="4" t="s">
+      <c r="H1" s="3"/>
+      <c r="I1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="L1" s="4"/>
-    </row>
-    <row r="2" ht="13" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="J1" s="4"/>
+    </row>
+    <row r="2" ht="14" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="1"/>
       <c r="B2" s="1"/>
-      <c r="C2" s="1"/>
+      <c r="C2" s="2"/>
       <c r="D2" s="2"/>
       <c r="E2" s="2"/>
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
-      <c r="H2" s="2"/>
-      <c r="I2" s="2"/>
-      <c r="J2" s="3"/>
-      <c r="K2" s="4"/>
-      <c r="L2" s="4"/>
-    </row>
-    <row r="3" ht="13" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="H2" s="3"/>
+      <c r="I2" s="4"/>
+      <c r="J2" s="4"/>
+    </row>
+    <row r="3" ht="14" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
       <c r="B3" s="1"/>
-      <c r="C3" s="1"/>
+      <c r="C3" s="2"/>
       <c r="D3" s="2"/>
       <c r="E3" s="2"/>
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
-      <c r="H3" s="2"/>
-      <c r="I3" s="2"/>
-      <c r="J3" s="3"/>
-      <c r="K3" s="4"/>
-      <c r="L3" s="4"/>
-    </row>
-    <row r="4" ht="14" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="H3" s="3"/>
+      <c r="I3" s="4"/>
+      <c r="J3" s="4"/>
+    </row>
+    <row r="4" ht="13" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
         <v>3</v>
       </c>
       <c r="B4" s="5"/>
-      <c r="C4" s="5"/>
-      <c r="D4" s="6" t="s">
+      <c r="C4" s="6" t="s">
         <v>4</v>
       </c>
+      <c r="D4" s="6"/>
       <c r="E4" s="6"/>
       <c r="F4" s="6"/>
       <c r="G4" s="6"/>
       <c r="H4" s="6"/>
-      <c r="I4" s="6"/>
-      <c r="J4" s="6"/>
-      <c r="K4" s="7" t="s">
+      <c r="I4" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="L4" s="7"/>
-    </row>
-    <row r="5" ht="26" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="J4" s="7"/>
+    </row>
+    <row r="5" ht="32" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" s="8"/>
       <c r="B5" s="8"/>
       <c r="C5" s="8"/>
@@ -3231,10 +3179,8 @@
       <c r="H5" s="8"/>
       <c r="I5" s="8"/>
       <c r="J5" s="8"/>
-      <c r="K5" s="8"/>
-      <c r="L5" s="8"/>
-    </row>
-    <row r="6" ht="22" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="6" ht="22" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
         <v>6</v>
       </c>
@@ -3257,1188 +3203,1055 @@
         <v>12</v>
       </c>
       <c r="H6" s="11"/>
-      <c r="I6" s="11"/>
-      <c r="J6" s="12" t="s">
+      <c r="I6" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="K6" s="12"/>
-      <c r="L6" s="12"/>
-    </row>
-    <row r="7" ht="17" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="J6" s="12"/>
+    </row>
+    <row r="7" ht="16" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" s="9"/>
       <c r="B7" s="13" t="s">
         <v>14</v>
       </c>
-      <c r="C7" s="13"/>
+      <c r="C7" s="13" t="s">
+        <v>15</v>
+      </c>
       <c r="D7" s="13" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E7" s="13" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F7" s="13" t="s">
-        <v>17</v>
-      </c>
-      <c r="G7" s="13" t="s">
         <v>18</v>
       </c>
-      <c r="H7" s="13"/>
-      <c r="I7" s="14" t="s">
+      <c r="G7" s="14"/>
+      <c r="H7" s="14"/>
+      <c r="I7" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="J7" s="14"/>
-      <c r="K7" s="14"/>
-      <c r="L7" s="14"/>
-    </row>
-    <row r="8" ht="18" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A8" s="15" t="s">
+      <c r="J7" s="15"/>
+    </row>
+    <row r="8" ht="18" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A8" s="16" t="s">
         <v>20</v>
       </c>
-      <c r="B8" s="16" t="s">
+      <c r="B8" s="17" t="s">
         <v>21</v>
       </c>
-      <c r="C8" s="16"/>
-      <c r="D8" s="16"/>
-      <c r="E8" s="16" t="s">
+      <c r="C8" s="17"/>
+      <c r="D8" s="17" t="s">
         <v>22</v>
       </c>
-      <c r="F8" s="16"/>
-      <c r="G8" s="16"/>
-      <c r="H8" s="17" t="s">
+      <c r="E8" s="17"/>
+      <c r="F8" s="17"/>
+      <c r="G8" s="18" t="s">
         <v>23</v>
       </c>
-      <c r="I8" s="17"/>
-      <c r="J8" s="17"/>
-      <c r="K8" s="17"/>
-      <c r="L8" s="17"/>
-    </row>
-    <row r="9" ht="30" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A9" s="18"/>
-      <c r="B9" s="19" t="s">
+      <c r="H8" s="18"/>
+      <c r="I8" s="18"/>
+      <c r="J8" s="19"/>
+    </row>
+    <row r="9" ht="32" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A9" s="20" t="s">
         <v>24</v>
       </c>
-      <c r="C9" s="20" t="s">
+      <c r="B9" s="21" t="s">
         <v>25</v>
       </c>
-      <c r="D9" s="20"/>
-      <c r="E9" s="21" t="s">
+      <c r="C9" s="21"/>
+      <c r="D9" s="22" t="s">
         <v>26</v>
       </c>
-      <c r="F9" s="21"/>
-      <c r="G9" s="20" t="s">
+      <c r="E9" s="22"/>
+      <c r="F9" s="21" t="s">
         <v>27</v>
       </c>
-      <c r="H9" s="20"/>
-      <c r="I9" s="20" t="s">
+      <c r="G9" s="21"/>
+      <c r="H9" s="21" t="s">
         <v>28</v>
       </c>
-      <c r="J9" s="20"/>
-      <c r="K9" s="22" t="s">
+      <c r="I9" s="21"/>
+      <c r="J9" s="23" t="s">
         <v>29</v>
       </c>
-      <c r="L9" s="22"/>
-    </row>
-    <row r="10" ht="18" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A10" s="23" t="s">
+    </row>
+    <row r="10" ht="18" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A10" s="24" t="s">
         <v>30</v>
       </c>
-      <c r="B10" s="24" t="s">
+      <c r="B10" s="25" t="s">
         <v>31</v>
       </c>
-      <c r="C10" s="25" t="s">
+      <c r="C10" s="26">
+        <v>145000000</v>
+      </c>
+      <c r="D10" s="25" t="s">
         <v>32</v>
       </c>
-      <c r="D10" s="26">
-        <v>145000000</v>
-      </c>
-      <c r="E10" s="25" t="s">
+      <c r="E10" s="26">
+        <v>0</v>
+      </c>
+      <c r="F10" s="25" t="s">
         <v>33</v>
       </c>
-      <c r="F10" s="26">
-        <v>0</v>
-      </c>
-      <c r="G10" s="25" t="s">
+      <c r="G10" s="26">
+        <v>18500000</v>
+      </c>
+      <c r="H10" s="25" t="s">
         <v>34</v>
       </c>
-      <c r="H10" s="26">
-        <v>18500000</v>
-      </c>
-      <c r="I10" s="25" t="s">
+      <c r="I10" s="26">
+        <v>0</v>
+      </c>
+      <c r="J10" s="27" t="s">
         <v>35</v>
       </c>
-      <c r="J10" s="26">
-        <v>0</v>
-      </c>
-      <c r="K10" s="27" t="s">
+    </row>
+    <row r="11" ht="18" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A11" s="28" t="s">
         <v>36</v>
       </c>
-      <c r="L10" s="27"/>
-    </row>
-    <row r="11" ht="18" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A11" s="23"/>
-      <c r="B11" s="28" t="s">
-        <v>37</v>
-      </c>
+      <c r="B11" s="29"/>
       <c r="C11" s="29"/>
       <c r="D11" s="29"/>
       <c r="E11" s="29"/>
       <c r="F11" s="29"/>
       <c r="G11" s="29"/>
-      <c r="H11" s="29"/>
-      <c r="I11" s="30" t="s">
+      <c r="H11" s="30" t="s">
+        <v>37</v>
+      </c>
+      <c r="I11" s="31">
+        <v>0</v>
+      </c>
+      <c r="J11" s="27" t="s">
         <v>38</v>
       </c>
-      <c r="J11" s="31">
-        <v>0</v>
-      </c>
-      <c r="K11" s="27" t="s">
+    </row>
+    <row r="12" ht="18" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A12" s="24" t="s">
         <v>39</v>
       </c>
-      <c r="L11" s="27"/>
-    </row>
-    <row r="12" ht="18" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A12" s="23"/>
-      <c r="B12" s="24" t="s">
+      <c r="B12" s="25" t="s">
         <v>40</v>
       </c>
-      <c r="C12" s="25" t="s">
+      <c r="C12" s="26">
+        <v>11600000</v>
+      </c>
+      <c r="D12" s="25" t="s">
         <v>41</v>
       </c>
-      <c r="D12" s="26">
-        <v>11600000</v>
-      </c>
-      <c r="E12" s="25" t="s">
+      <c r="E12" s="26">
+        <v>0</v>
+      </c>
+      <c r="F12" s="25" t="s">
         <v>42</v>
       </c>
-      <c r="F12" s="26">
-        <v>0</v>
-      </c>
-      <c r="G12" s="25" t="s">
+      <c r="G12" s="26">
+        <v>2100000</v>
+      </c>
+      <c r="H12" s="25" t="s">
         <v>43</v>
       </c>
-      <c r="H12" s="26">
-        <v>2100000</v>
-      </c>
-      <c r="I12" s="25" t="s">
+      <c r="I12" s="26">
+        <v>0</v>
+      </c>
+      <c r="J12" s="27" t="s">
         <v>44</v>
       </c>
-      <c r="J12" s="26">
-        <v>0</v>
-      </c>
-      <c r="K12" s="27" t="s">
+    </row>
+    <row r="13" ht="18" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A13" s="28" t="s">
         <v>45</v>
       </c>
-      <c r="L12" s="27"/>
-    </row>
-    <row r="13" ht="18" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A13" s="23"/>
-      <c r="B13" s="28" t="s">
+      <c r="B13" s="29"/>
+      <c r="C13" s="29"/>
+      <c r="D13" s="30" t="s">
         <v>46</v>
       </c>
-      <c r="C13" s="29"/>
-      <c r="D13" s="29"/>
-      <c r="E13" s="30" t="s">
+      <c r="E13" s="31">
+        <v>0</v>
+      </c>
+      <c r="F13" s="30" t="s">
         <v>47</v>
       </c>
-      <c r="F13" s="31">
-        <v>0</v>
-      </c>
-      <c r="G13" s="30" t="s">
+      <c r="G13" s="31">
+        <v>3500000</v>
+      </c>
+      <c r="H13" s="30" t="s">
         <v>48</v>
       </c>
-      <c r="H13" s="31">
-        <v>3500000</v>
-      </c>
-      <c r="I13" s="30" t="s">
+      <c r="I13" s="31">
+        <v>0</v>
+      </c>
+      <c r="J13" s="27" t="s">
         <v>49</v>
       </c>
-      <c r="J13" s="31">
-        <v>0</v>
-      </c>
-      <c r="K13" s="27" t="s">
+    </row>
+    <row r="14" ht="18" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A14" s="24" t="s">
         <v>50</v>
       </c>
-      <c r="L13" s="27"/>
-    </row>
-    <row r="14" ht="18" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A14" s="23"/>
-      <c r="B14" s="24" t="s">
+      <c r="B14" s="25" t="s">
         <v>51</v>
       </c>
-      <c r="C14" s="25" t="s">
+      <c r="C14" s="26">
+        <v>133400000</v>
+      </c>
+      <c r="D14" s="25" t="s">
         <v>52</v>
       </c>
-      <c r="D14" s="26">
-        <v>133400000</v>
-      </c>
-      <c r="E14" s="25" t="s">
+      <c r="E14" s="26">
+        <v>0</v>
+      </c>
+      <c r="F14" s="25" t="s">
         <v>53</v>
       </c>
-      <c r="F14" s="26">
-        <v>0</v>
-      </c>
-      <c r="G14" s="25" t="s">
+      <c r="G14" s="26">
+        <v>12900000</v>
+      </c>
+      <c r="H14" s="25" t="s">
         <v>54</v>
       </c>
-      <c r="H14" s="26">
-        <v>12900000</v>
-      </c>
-      <c r="I14" s="25" t="s">
+      <c r="I14" s="26">
+        <v>0</v>
+      </c>
+      <c r="J14" s="27" t="s">
         <v>55</v>
       </c>
-      <c r="J14" s="26">
-        <v>0</v>
-      </c>
-      <c r="K14" s="27" t="s">
+    </row>
+    <row r="15" ht="18" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A15" s="28" t="s">
         <v>56</v>
       </c>
-      <c r="L14" s="27"/>
-    </row>
-    <row r="15" ht="18" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A15" s="23"/>
-      <c r="B15" s="28" t="s">
-        <v>57</v>
-      </c>
+      <c r="B15" s="29"/>
       <c r="C15" s="29"/>
       <c r="D15" s="29"/>
       <c r="E15" s="29"/>
-      <c r="F15" s="29"/>
-      <c r="G15" s="30" t="s">
+      <c r="F15" s="30" t="s">
+        <v>57</v>
+      </c>
+      <c r="G15" s="31">
+        <v>0</v>
+      </c>
+      <c r="H15" s="30" t="s">
         <v>58</v>
       </c>
-      <c r="H15" s="31">
-        <v>0</v>
-      </c>
-      <c r="I15" s="30" t="s">
+      <c r="I15" s="31">
+        <v>0</v>
+      </c>
+      <c r="J15" s="32" t="s">
         <v>59</v>
       </c>
-      <c r="J15" s="31">
-        <v>0</v>
-      </c>
-      <c r="K15" s="32" t="s">
+    </row>
+    <row r="16" ht="18" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A16" s="24" t="s">
         <v>60</v>
       </c>
-      <c r="L15" s="32"/>
-    </row>
-    <row r="16" ht="18" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A16" s="23"/>
-      <c r="B16" s="33" t="s">
+      <c r="B16" s="25" t="s">
         <v>61</v>
       </c>
-      <c r="C16" s="34" t="s">
+      <c r="C16" s="26">
+        <v>12000000</v>
+      </c>
+      <c r="D16" s="25" t="s">
         <v>62</v>
       </c>
-      <c r="D16" s="35">
-        <v>12000000</v>
-      </c>
-      <c r="E16" s="34" t="s">
+      <c r="E16" s="26">
+        <v>0</v>
+      </c>
+      <c r="F16" s="25" t="s">
         <v>63</v>
       </c>
-      <c r="F16" s="35">
-        <v>0</v>
-      </c>
-      <c r="G16" s="34" t="s">
+      <c r="G16" s="26">
+        <v>0</v>
+      </c>
+      <c r="H16" s="25" t="s">
         <v>64</v>
       </c>
-      <c r="H16" s="35">
-        <v>0</v>
-      </c>
-      <c r="I16" s="34" t="s">
+      <c r="I16" s="26">
+        <v>0</v>
+      </c>
+      <c r="J16" s="33" t="s">
         <v>65</v>
       </c>
-      <c r="J16" s="35">
-        <v>0</v>
-      </c>
-      <c r="K16" s="36" t="s">
+    </row>
+    <row r="17" ht="18" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A17" s="34" t="s">
         <v>66</v>
       </c>
-      <c r="L16" s="36"/>
-    </row>
-    <row r="17" ht="18" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A17" s="23"/>
-      <c r="B17" s="33" t="s">
+      <c r="B17" s="35" t="s">
         <v>67</v>
       </c>
-      <c r="C17" s="34" t="s">
+      <c r="C17" s="36">
+        <v>26500000</v>
+      </c>
+      <c r="D17" s="35" t="s">
         <v>68</v>
       </c>
-      <c r="D17" s="35">
-        <v>26500000</v>
-      </c>
-      <c r="E17" s="34" t="s">
+      <c r="E17" s="36">
+        <v>0</v>
+      </c>
+      <c r="F17" s="35" t="s">
         <v>69</v>
       </c>
-      <c r="F17" s="35">
-        <v>0</v>
-      </c>
-      <c r="G17" s="34" t="s">
+      <c r="G17" s="36">
+        <v>0</v>
+      </c>
+      <c r="H17" s="35" t="s">
         <v>70</v>
       </c>
-      <c r="H17" s="35">
-        <v>0</v>
-      </c>
-      <c r="I17" s="34" t="s">
+      <c r="I17" s="36">
+        <v>0</v>
+      </c>
+      <c r="J17" s="27" t="s">
         <v>71</v>
       </c>
-      <c r="J17" s="35">
-        <v>0</v>
-      </c>
-      <c r="K17" s="27" t="s">
+    </row>
+    <row r="18" ht="18" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A18" s="34" t="s">
         <v>72</v>
       </c>
-      <c r="L17" s="27"/>
-    </row>
-    <row r="18" ht="18" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A18" s="23"/>
-      <c r="B18" s="33" t="s">
+      <c r="B18" s="35" t="s">
         <v>73</v>
       </c>
-      <c r="C18" s="34" t="s">
+      <c r="C18" s="36">
+        <v>38500000</v>
+      </c>
+      <c r="D18" s="35" t="s">
         <v>74</v>
       </c>
-      <c r="D18" s="35">
-        <v>38500000</v>
-      </c>
-      <c r="E18" s="34" t="s">
+      <c r="E18" s="36">
+        <v>0</v>
+      </c>
+      <c r="F18" s="35" t="s">
         <v>75</v>
       </c>
-      <c r="F18" s="35">
-        <v>0</v>
-      </c>
-      <c r="G18" s="34" t="s">
+      <c r="G18" s="36">
+        <v>0</v>
+      </c>
+      <c r="H18" s="35" t="s">
         <v>76</v>
       </c>
-      <c r="H18" s="35">
-        <v>0</v>
-      </c>
-      <c r="I18" s="34" t="s">
+      <c r="I18" s="36">
+        <v>0</v>
+      </c>
+      <c r="J18" s="27" t="s">
         <v>77</v>
       </c>
-      <c r="J18" s="35">
-        <v>0</v>
-      </c>
-      <c r="K18" s="27" t="s">
+    </row>
+    <row r="19" ht="18" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A19" s="28" t="s">
         <v>78</v>
       </c>
-      <c r="L18" s="27"/>
-    </row>
-    <row r="19" ht="18" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A19" s="23"/>
-      <c r="B19" s="37" t="s">
+      <c r="B19" s="30" t="s">
         <v>79</v>
       </c>
-      <c r="C19" s="38" t="s">
+      <c r="C19" s="31">
+        <v>8400000</v>
+      </c>
+      <c r="D19" s="30" t="s">
         <v>80</v>
       </c>
-      <c r="D19" s="39">
-        <v>8400000</v>
-      </c>
-      <c r="E19" s="38" t="s">
+      <c r="E19" s="31">
+        <v>0</v>
+      </c>
+      <c r="F19" s="30" t="s">
         <v>81</v>
       </c>
-      <c r="F19" s="39">
-        <v>0</v>
-      </c>
-      <c r="G19" s="38" t="s">
+      <c r="G19" s="31">
+        <v>0</v>
+      </c>
+      <c r="H19" s="30" t="s">
         <v>82</v>
       </c>
-      <c r="H19" s="39">
-        <v>0</v>
-      </c>
-      <c r="I19" s="38" t="s">
+      <c r="I19" s="31">
+        <v>0</v>
+      </c>
+      <c r="J19" s="27" t="s">
         <v>83</v>
       </c>
-      <c r="J19" s="39">
-        <v>0</v>
-      </c>
-      <c r="K19" s="27" t="s">
+    </row>
+    <row r="20" ht="18" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A20" s="24" t="s">
         <v>84</v>
       </c>
-      <c r="L19" s="27"/>
-    </row>
-    <row r="20" ht="18" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A20" s="23"/>
-      <c r="B20" s="37" t="s">
+      <c r="B20" s="25" t="s">
         <v>85</v>
       </c>
-      <c r="C20" s="38" t="s">
+      <c r="C20" s="26">
+        <v>6460000</v>
+      </c>
+      <c r="D20" s="25" t="s">
         <v>86</v>
       </c>
-      <c r="D20" s="39">
-        <v>6460000</v>
-      </c>
-      <c r="E20" s="38" t="s">
+      <c r="E20" s="26">
+        <v>0</v>
+      </c>
+      <c r="F20" s="25" t="s">
         <v>87</v>
       </c>
-      <c r="F20" s="39">
-        <v>0</v>
-      </c>
-      <c r="G20" s="38" t="s">
+      <c r="G20" s="26">
+        <v>520000</v>
+      </c>
+      <c r="H20" s="25" t="s">
         <v>88</v>
       </c>
-      <c r="H20" s="39">
+      <c r="I20" s="26">
+        <v>0</v>
+      </c>
+      <c r="J20" s="32" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="21" ht="18" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A21" s="28" t="s">
+        <v>90</v>
+      </c>
+      <c r="B21" s="30" t="s">
+        <v>91</v>
+      </c>
+      <c r="C21" s="31">
+        <v>14860000</v>
+      </c>
+      <c r="D21" s="30" t="s">
+        <v>92</v>
+      </c>
+      <c r="E21" s="31">
+        <v>0</v>
+      </c>
+      <c r="F21" s="30" t="s">
+        <v>93</v>
+      </c>
+      <c r="G21" s="31">
         <v>520000</v>
       </c>
-      <c r="I20" s="38" t="s">
-        <v>89</v>
-      </c>
-      <c r="J20" s="39">
-        <v>0</v>
-      </c>
-      <c r="K20" s="32" t="s">
-        <v>90</v>
-      </c>
-      <c r="L20" s="32"/>
-    </row>
-    <row r="21" ht="18" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A21" s="23"/>
-      <c r="B21" s="37" t="s">
-        <v>91</v>
-      </c>
-      <c r="C21" s="38" t="s">
-        <v>92</v>
-      </c>
-      <c r="D21" s="39">
-        <v>14860000</v>
-      </c>
-      <c r="E21" s="38" t="s">
-        <v>93</v>
-      </c>
-      <c r="F21" s="39">
-        <v>0</v>
-      </c>
-      <c r="G21" s="38" t="s">
+      <c r="H21" s="30" t="s">
         <v>94</v>
       </c>
-      <c r="H21" s="39">
+      <c r="I21" s="31">
+        <v>0</v>
+      </c>
+      <c r="J21" s="32" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="22" ht="18" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A22" s="24" t="s">
+        <v>96</v>
+      </c>
+      <c r="B22" s="25" t="s">
+        <v>97</v>
+      </c>
+      <c r="C22" s="26">
+        <v>48720000</v>
+      </c>
+      <c r="D22" s="25" t="s">
+        <v>98</v>
+      </c>
+      <c r="E22" s="26">
+        <v>0</v>
+      </c>
+      <c r="F22" s="25" t="s">
+        <v>99</v>
+      </c>
+      <c r="G22" s="26">
         <v>520000</v>
       </c>
-      <c r="I21" s="38" t="s">
-        <v>95</v>
-      </c>
-      <c r="J21" s="39">
-        <v>0</v>
-      </c>
-      <c r="K21" s="32" t="s">
-        <v>96</v>
-      </c>
-      <c r="L21" s="32"/>
-    </row>
-    <row r="22" ht="18" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A22" s="23"/>
-      <c r="B22" s="24" t="s">
-        <v>97</v>
-      </c>
-      <c r="C22" s="25" t="s">
-        <v>98</v>
-      </c>
-      <c r="D22" s="26">
-        <v>48720000</v>
-      </c>
-      <c r="E22" s="25" t="s">
-        <v>99</v>
-      </c>
-      <c r="F22" s="26">
-        <v>0</v>
-      </c>
-      <c r="G22" s="25" t="s">
+      <c r="H22" s="25" t="s">
         <v>100</v>
       </c>
-      <c r="H22" s="26">
-        <v>520000</v>
-      </c>
-      <c r="I22" s="25" t="s">
+      <c r="I22" s="26">
+        <v>0</v>
+      </c>
+      <c r="J22" s="27" t="s">
         <v>101</v>
       </c>
-      <c r="J22" s="26">
-        <v>0</v>
-      </c>
-      <c r="K22" s="27" t="s">
+    </row>
+    <row r="23" ht="18" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A23" s="28" t="s">
         <v>102</v>
       </c>
-      <c r="L22" s="27"/>
-    </row>
-    <row r="23" ht="18" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A23" s="23"/>
-      <c r="B23" s="28" t="s">
+      <c r="B23" s="29"/>
+      <c r="C23" s="29"/>
+      <c r="D23" s="30" t="s">
         <v>103</v>
       </c>
-      <c r="C23" s="29"/>
-      <c r="D23" s="29"/>
-      <c r="E23" s="30" t="s">
+      <c r="E23" s="31">
+        <v>0</v>
+      </c>
+      <c r="F23" s="30" t="s">
         <v>104</v>
       </c>
-      <c r="F23" s="31">
-        <v>0</v>
-      </c>
-      <c r="G23" s="30" t="s">
+      <c r="G23" s="31">
+        <v>12380000</v>
+      </c>
+      <c r="H23" s="30" t="s">
         <v>105</v>
       </c>
-      <c r="H23" s="31">
+      <c r="I23" s="31">
+        <v>0</v>
+      </c>
+      <c r="J23" s="27" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="24" ht="18" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A24" s="24" t="s">
+        <v>107</v>
+      </c>
+      <c r="B24" s="29"/>
+      <c r="C24" s="29"/>
+      <c r="D24" s="25" t="s">
+        <v>108</v>
+      </c>
+      <c r="E24" s="26">
+        <v>0</v>
+      </c>
+      <c r="F24" s="25" t="s">
+        <v>109</v>
+      </c>
+      <c r="G24" s="26">
+        <v>0</v>
+      </c>
+      <c r="H24" s="25" t="s">
+        <v>110</v>
+      </c>
+      <c r="I24" s="26">
+        <v>0</v>
+      </c>
+      <c r="J24" s="32" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="25" ht="18" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A25" s="28" t="s">
+        <v>112</v>
+      </c>
+      <c r="B25" s="29"/>
+      <c r="C25" s="29"/>
+      <c r="D25" s="30" t="s">
+        <v>113</v>
+      </c>
+      <c r="E25" s="31">
+        <v>0</v>
+      </c>
+      <c r="F25" s="30" t="s">
+        <v>114</v>
+      </c>
+      <c r="G25" s="31">
+        <v>0</v>
+      </c>
+      <c r="H25" s="30" t="s">
+        <v>115</v>
+      </c>
+      <c r="I25" s="31">
+        <v>0</v>
+      </c>
+      <c r="J25" s="27" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="26" ht="18" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A26" s="24" t="s">
+        <v>117</v>
+      </c>
+      <c r="B26" s="25" t="s">
+        <v>118</v>
+      </c>
+      <c r="C26" s="26">
+        <v>84680000</v>
+      </c>
+      <c r="D26" s="25" t="s">
+        <v>119</v>
+      </c>
+      <c r="E26" s="26">
+        <v>0</v>
+      </c>
+      <c r="F26" s="25" t="s">
+        <v>120</v>
+      </c>
+      <c r="G26" s="26">
         <v>12380000</v>
       </c>
-      <c r="I23" s="30" t="s">
-        <v>106</v>
-      </c>
-      <c r="J23" s="31">
-        <v>0</v>
-      </c>
-      <c r="K23" s="27" t="s">
-        <v>107</v>
-      </c>
-      <c r="L23" s="27"/>
-    </row>
-    <row r="24" ht="18" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A24" s="23"/>
-      <c r="B24" s="24" t="s">
-        <v>108</v>
-      </c>
-      <c r="C24" s="29"/>
-      <c r="D24" s="29"/>
-      <c r="E24" s="25" t="s">
-        <v>109</v>
-      </c>
-      <c r="F24" s="26">
-        <v>0</v>
-      </c>
-      <c r="G24" s="25" t="s">
-        <v>110</v>
-      </c>
-      <c r="H24" s="26">
-        <v>0</v>
-      </c>
-      <c r="I24" s="25" t="s">
-        <v>111</v>
-      </c>
-      <c r="J24" s="26">
-        <v>0</v>
-      </c>
-      <c r="K24" s="32" t="s">
-        <v>112</v>
-      </c>
-      <c r="L24" s="32"/>
-    </row>
-    <row r="25" ht="18" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A25" s="23"/>
-      <c r="B25" s="28" t="s">
-        <v>113</v>
-      </c>
-      <c r="C25" s="29"/>
-      <c r="D25" s="29"/>
-      <c r="E25" s="30" t="s">
-        <v>114</v>
-      </c>
-      <c r="F25" s="31">
-        <v>0</v>
-      </c>
-      <c r="G25" s="30" t="s">
-        <v>115</v>
-      </c>
-      <c r="H25" s="31">
-        <v>0</v>
-      </c>
-      <c r="I25" s="30" t="s">
-        <v>116</v>
-      </c>
-      <c r="J25" s="31">
-        <v>0</v>
-      </c>
-      <c r="K25" s="27" t="s">
-        <v>117</v>
-      </c>
-      <c r="L25" s="27"/>
-    </row>
-    <row r="26" ht="18" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A26" s="23"/>
-      <c r="B26" s="24" t="s">
-        <v>118</v>
-      </c>
-      <c r="C26" s="25" t="s">
-        <v>119</v>
-      </c>
-      <c r="D26" s="26">
-        <v>84680000</v>
-      </c>
-      <c r="E26" s="25" t="s">
-        <v>120</v>
-      </c>
-      <c r="F26" s="26">
-        <v>0</v>
-      </c>
-      <c r="G26" s="25" t="s">
+      <c r="H26" s="25" t="s">
         <v>121</v>
       </c>
-      <c r="H26" s="26">
-        <v>12380000</v>
-      </c>
-      <c r="I26" s="25" t="s">
+      <c r="I26" s="26">
+        <v>0</v>
+      </c>
+      <c r="J26" s="27" t="s">
         <v>122</v>
       </c>
-      <c r="J26" s="26">
-        <v>0</v>
-      </c>
-      <c r="K26" s="27" t="s">
+    </row>
+    <row r="27" ht="17" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A27" s="37" t="s">
         <v>123</v>
       </c>
-      <c r="L26" s="27"/>
-    </row>
-    <row r="27" ht="17" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A27" s="18"/>
-      <c r="B27" s="40" t="s">
+      <c r="B27" s="37"/>
+      <c r="C27" s="37" t="s">
         <v>124</v>
       </c>
-      <c r="C27" s="40"/>
-      <c r="D27" s="40" t="s">
+      <c r="D27" s="37"/>
+      <c r="E27" s="38" t="s">
         <v>125</v>
       </c>
-      <c r="E27" s="40"/>
-      <c r="F27" s="41" t="s">
+      <c r="F27" s="38"/>
+      <c r="G27" s="37" t="s">
         <v>126</v>
       </c>
-      <c r="G27" s="41"/>
-      <c r="H27" s="40" t="s">
+      <c r="H27" s="37"/>
+      <c r="I27" s="39"/>
+      <c r="J27" s="40" t="s">
         <v>127</v>
       </c>
-      <c r="I27" s="40"/>
-      <c r="J27" s="42"/>
-      <c r="K27" s="43" t="s">
+    </row>
+    <row r="28" ht="17" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A28" s="37" t="s">
         <v>128</v>
       </c>
-      <c r="L27" s="43"/>
-    </row>
-    <row r="28" ht="17" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A28" s="44"/>
-      <c r="B28" s="40" t="s">
+      <c r="B28" s="37"/>
+      <c r="C28" s="37" t="s">
         <v>129</v>
       </c>
-      <c r="C28" s="40"/>
-      <c r="D28" s="40" t="s">
+      <c r="D28" s="37"/>
+      <c r="E28" s="38" t="s">
         <v>130</v>
       </c>
-      <c r="E28" s="40"/>
-      <c r="F28" s="41" t="s">
+      <c r="F28" s="38"/>
+      <c r="G28" s="37" t="s">
         <v>131</v>
       </c>
-      <c r="G28" s="41"/>
-      <c r="H28" s="40" t="s">
+      <c r="H28" s="37"/>
+      <c r="I28" s="39"/>
+      <c r="J28" s="40" t="s">
         <v>132</v>
       </c>
-      <c r="I28" s="40"/>
-      <c r="J28" s="42"/>
-      <c r="K28" s="43" t="s">
+    </row>
+    <row r="29" ht="17" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A29" s="41" t="s">
         <v>133</v>
       </c>
-      <c r="L28" s="43"/>
-    </row>
-    <row r="29" ht="17" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A29" s="45" t="s">
+      <c r="B29" s="41"/>
+      <c r="C29" s="41"/>
+      <c r="D29" s="41"/>
+      <c r="E29" s="41"/>
+      <c r="F29" s="41"/>
+      <c r="G29" s="41"/>
+      <c r="H29" s="41"/>
+      <c r="I29" s="41"/>
+      <c r="J29" s="42" t="s">
         <v>134</v>
       </c>
-      <c r="B29" s="45"/>
-      <c r="C29" s="45"/>
-      <c r="D29" s="45"/>
-      <c r="E29" s="45"/>
-      <c r="F29" s="45"/>
-      <c r="G29" s="45"/>
-      <c r="H29" s="45"/>
-      <c r="I29" s="45"/>
-      <c r="J29" s="45"/>
-      <c r="K29" s="46" t="s">
+    </row>
+    <row r="30" ht="17" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A30" s="43" t="s">
         <v>135</v>
       </c>
-      <c r="L29" s="46"/>
-    </row>
-    <row r="30" ht="17" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A30" s="47" t="s">
+      <c r="B30" s="43"/>
+      <c r="C30" s="43"/>
+      <c r="D30" s="44">
+        <v>0</v>
+      </c>
+      <c r="E30" s="44"/>
+      <c r="F30" s="44"/>
+      <c r="G30" s="44"/>
+      <c r="H30" s="44"/>
+      <c r="I30" s="44"/>
+      <c r="J30" s="40" t="s">
         <v>136</v>
       </c>
-      <c r="B30" s="47"/>
-      <c r="C30" s="47"/>
-      <c r="D30" s="48">
-        <v>0</v>
-      </c>
-      <c r="E30" s="48"/>
-      <c r="F30" s="48"/>
-      <c r="G30" s="48"/>
-      <c r="H30" s="48"/>
-      <c r="I30" s="48"/>
-      <c r="J30" s="48"/>
-      <c r="K30" s="43" t="s">
+    </row>
+    <row r="31" ht="17" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A31" s="43" t="s">
         <v>137</v>
       </c>
-      <c r="L30" s="43"/>
-    </row>
-    <row r="31" ht="17" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A31" s="47" t="s">
+      <c r="B31" s="43"/>
+      <c r="C31" s="43"/>
+      <c r="D31" s="44">
+        <v>0</v>
+      </c>
+      <c r="E31" s="44"/>
+      <c r="F31" s="44"/>
+      <c r="G31" s="44"/>
+      <c r="H31" s="44"/>
+      <c r="I31" s="44"/>
+      <c r="J31" s="40" t="s">
         <v>138</v>
       </c>
-      <c r="B31" s="47"/>
-      <c r="C31" s="47"/>
-      <c r="D31" s="48">
-        <v>0</v>
-      </c>
-      <c r="E31" s="48"/>
-      <c r="F31" s="48"/>
-      <c r="G31" s="48"/>
-      <c r="H31" s="48"/>
-      <c r="I31" s="48"/>
-      <c r="J31" s="48"/>
-      <c r="K31" s="43" t="s">
+    </row>
+    <row r="32" ht="17" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A32" s="43" t="s">
         <v>139</v>
       </c>
-      <c r="L31" s="43"/>
-    </row>
-    <row r="32" ht="17" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A32" s="47" t="s">
+      <c r="B32" s="43"/>
+      <c r="C32" s="43"/>
+      <c r="D32" s="44">
+        <v>0</v>
+      </c>
+      <c r="E32" s="44"/>
+      <c r="F32" s="44"/>
+      <c r="G32" s="44"/>
+      <c r="H32" s="44"/>
+      <c r="I32" s="44"/>
+      <c r="J32" s="45" t="s">
         <v>140</v>
       </c>
-      <c r="B32" s="47"/>
-      <c r="C32" s="47"/>
-      <c r="D32" s="48">
-        <v>0</v>
-      </c>
-      <c r="E32" s="48"/>
-      <c r="F32" s="48"/>
-      <c r="G32" s="48"/>
-      <c r="H32" s="48"/>
-      <c r="I32" s="48"/>
-      <c r="J32" s="48"/>
-      <c r="K32" s="49" t="s">
+    </row>
+    <row r="33" ht="17" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A33" s="43" t="s">
         <v>141</v>
       </c>
-      <c r="L32" s="49"/>
-    </row>
-    <row r="33" ht="17" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A33" s="47" t="s">
+      <c r="B33" s="43"/>
+      <c r="C33" s="43"/>
+      <c r="D33" s="44">
+        <v>0</v>
+      </c>
+      <c r="E33" s="44"/>
+      <c r="F33" s="44"/>
+      <c r="G33" s="44"/>
+      <c r="H33" s="44"/>
+      <c r="I33" s="44"/>
+      <c r="J33" s="46" t="s">
         <v>142</v>
       </c>
-      <c r="B33" s="47"/>
-      <c r="C33" s="47"/>
-      <c r="D33" s="48">
-        <v>0</v>
-      </c>
-      <c r="E33" s="48"/>
-      <c r="F33" s="48"/>
-      <c r="G33" s="48"/>
-      <c r="H33" s="48"/>
-      <c r="I33" s="48"/>
-      <c r="J33" s="48"/>
-      <c r="K33" s="50" t="s">
+    </row>
+    <row r="34" ht="17" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A34" s="47" t="s">
         <v>143</v>
       </c>
-      <c r="L33" s="50"/>
-    </row>
-    <row r="34" ht="17" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A34" s="51" t="s">
+      <c r="B34" s="47"/>
+      <c r="C34" s="47"/>
+      <c r="D34" s="48">
+        <v>0</v>
+      </c>
+      <c r="E34" s="48"/>
+      <c r="F34" s="48"/>
+      <c r="G34" s="48"/>
+      <c r="H34" s="48"/>
+      <c r="I34" s="48"/>
+      <c r="J34" s="40" t="s">
         <v>144</v>
       </c>
-      <c r="B34" s="51"/>
-      <c r="C34" s="51"/>
-      <c r="D34" s="52">
-        <v>0</v>
-      </c>
-      <c r="E34" s="52"/>
-      <c r="F34" s="52"/>
-      <c r="G34" s="52"/>
-      <c r="H34" s="52"/>
-      <c r="I34" s="52"/>
-      <c r="J34" s="52"/>
-      <c r="K34" s="43" t="s">
+    </row>
+    <row r="35" ht="17" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A35" s="41" t="s">
         <v>145</v>
       </c>
-      <c r="L34" s="43"/>
-    </row>
-    <row r="35" ht="17" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A35" s="45" t="s">
+      <c r="B35" s="41"/>
+      <c r="C35" s="41"/>
+      <c r="D35" s="41"/>
+      <c r="E35" s="41"/>
+      <c r="F35" s="41"/>
+      <c r="G35" s="41"/>
+      <c r="H35" s="41"/>
+      <c r="I35" s="41"/>
+      <c r="J35" s="40" t="s">
         <v>146</v>
       </c>
-      <c r="B35" s="45"/>
-      <c r="C35" s="45"/>
-      <c r="D35" s="45"/>
-      <c r="E35" s="45"/>
-      <c r="F35" s="45"/>
-      <c r="G35" s="45"/>
-      <c r="H35" s="45"/>
-      <c r="I35" s="45"/>
-      <c r="J35" s="45"/>
-      <c r="K35" s="43" t="s">
+    </row>
+    <row r="36" ht="17" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A36" s="43" t="s">
         <v>147</v>
       </c>
-      <c r="L35" s="43"/>
-    </row>
-    <row r="36" ht="17" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A36" s="47" t="s">
+      <c r="B36" s="43"/>
+      <c r="C36" s="43"/>
+      <c r="D36" s="44">
+        <v>0</v>
+      </c>
+      <c r="E36" s="44"/>
+      <c r="F36" s="44"/>
+      <c r="G36" s="44"/>
+      <c r="H36" s="44"/>
+      <c r="I36" s="44"/>
+      <c r="J36" s="40" t="s">
         <v>148</v>
       </c>
-      <c r="B36" s="47"/>
-      <c r="C36" s="47"/>
-      <c r="D36" s="48">
-        <v>0</v>
-      </c>
-      <c r="E36" s="48"/>
-      <c r="F36" s="48"/>
-      <c r="G36" s="48"/>
-      <c r="H36" s="48"/>
-      <c r="I36" s="48"/>
-      <c r="J36" s="48"/>
-      <c r="K36" s="43" t="s">
+    </row>
+    <row r="37" ht="17" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A37" s="43" t="s">
         <v>149</v>
       </c>
-      <c r="L36" s="43"/>
-    </row>
-    <row r="37" ht="17" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A37" s="47" t="s">
+      <c r="B37" s="43"/>
+      <c r="C37" s="43"/>
+      <c r="D37" s="44">
+        <v>0</v>
+      </c>
+      <c r="E37" s="44"/>
+      <c r="F37" s="44"/>
+      <c r="G37" s="44"/>
+      <c r="H37" s="44"/>
+      <c r="I37" s="44"/>
+      <c r="J37" s="40" t="s">
         <v>150</v>
       </c>
-      <c r="B37" s="47"/>
-      <c r="C37" s="47"/>
-      <c r="D37" s="48">
-        <v>0</v>
-      </c>
-      <c r="E37" s="48"/>
-      <c r="F37" s="48"/>
-      <c r="G37" s="48"/>
-      <c r="H37" s="48"/>
-      <c r="I37" s="48"/>
-      <c r="J37" s="48"/>
-      <c r="K37" s="43" t="s">
+    </row>
+    <row r="38" ht="17" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A38" s="43" t="s">
         <v>151</v>
       </c>
-      <c r="L37" s="43"/>
-    </row>
-    <row r="38" ht="17" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A38" s="47" t="s">
+      <c r="B38" s="43"/>
+      <c r="C38" s="43"/>
+      <c r="D38" s="44">
+        <v>0</v>
+      </c>
+      <c r="E38" s="44"/>
+      <c r="F38" s="44"/>
+      <c r="G38" s="44"/>
+      <c r="H38" s="44"/>
+      <c r="I38" s="44"/>
+      <c r="J38" s="42" t="s">
         <v>152</v>
       </c>
-      <c r="B38" s="47"/>
-      <c r="C38" s="47"/>
-      <c r="D38" s="48">
-        <v>0</v>
-      </c>
-      <c r="E38" s="48"/>
-      <c r="F38" s="48"/>
-      <c r="G38" s="48"/>
-      <c r="H38" s="48"/>
-      <c r="I38" s="48"/>
-      <c r="J38" s="48"/>
-      <c r="K38" s="46" t="s">
+    </row>
+    <row r="39" ht="17" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A39" s="43" t="s">
         <v>153</v>
       </c>
-      <c r="L38" s="46"/>
-    </row>
-    <row r="39" ht="17" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A39" s="47" t="s">
+      <c r="B39" s="43"/>
+      <c r="C39" s="43"/>
+      <c r="D39" s="44">
+        <v>4500000</v>
+      </c>
+      <c r="E39" s="44"/>
+      <c r="F39" s="44"/>
+      <c r="G39" s="44"/>
+      <c r="H39" s="44"/>
+      <c r="I39" s="44"/>
+      <c r="J39" s="49" t="s">
         <v>154</v>
       </c>
-      <c r="B39" s="47"/>
-      <c r="C39" s="47"/>
-      <c r="D39" s="48">
+    </row>
+    <row r="40" ht="17" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A40" s="43" t="s">
+        <v>155</v>
+      </c>
+      <c r="B40" s="43"/>
+      <c r="C40" s="43"/>
+      <c r="D40" s="44">
+        <v>0</v>
+      </c>
+      <c r="E40" s="44"/>
+      <c r="F40" s="44"/>
+      <c r="G40" s="44"/>
+      <c r="H40" s="44"/>
+      <c r="I40" s="44"/>
+      <c r="J40" s="40" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="41" ht="17" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A41" s="43" t="s">
+        <v>157</v>
+      </c>
+      <c r="B41" s="43"/>
+      <c r="C41" s="43"/>
+      <c r="D41" s="44">
+        <v>0</v>
+      </c>
+      <c r="E41" s="44"/>
+      <c r="F41" s="44"/>
+      <c r="G41" s="44"/>
+      <c r="H41" s="44"/>
+      <c r="I41" s="44"/>
+      <c r="J41" s="40" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="42" ht="17" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A42" s="43" t="s">
+        <v>159</v>
+      </c>
+      <c r="B42" s="43"/>
+      <c r="C42" s="43"/>
+      <c r="D42" s="44">
+        <v>0</v>
+      </c>
+      <c r="E42" s="44"/>
+      <c r="F42" s="44"/>
+      <c r="G42" s="44"/>
+      <c r="H42" s="44"/>
+      <c r="I42" s="44"/>
+      <c r="J42" s="40" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="43" ht="17" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A43" s="47" t="s">
+        <v>161</v>
+      </c>
+      <c r="B43" s="47"/>
+      <c r="C43" s="47"/>
+      <c r="D43" s="48">
         <v>4500000</v>
       </c>
-      <c r="E39" s="48"/>
-      <c r="F39" s="48"/>
-      <c r="G39" s="48"/>
-      <c r="H39" s="48"/>
-      <c r="I39" s="48"/>
-      <c r="J39" s="48"/>
-      <c r="K39" s="53" t="s">
-        <v>155</v>
-      </c>
-      <c r="L39" s="53"/>
-    </row>
-    <row r="40" ht="17" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A40" s="47" t="s">
-        <v>156</v>
-      </c>
-      <c r="B40" s="47"/>
-      <c r="C40" s="47"/>
-      <c r="D40" s="48">
-        <v>0</v>
-      </c>
-      <c r="E40" s="48"/>
-      <c r="F40" s="48"/>
-      <c r="G40" s="48"/>
-      <c r="H40" s="48"/>
-      <c r="I40" s="48"/>
-      <c r="J40" s="48"/>
-      <c r="K40" s="43" t="s">
-        <v>157</v>
-      </c>
-      <c r="L40" s="43"/>
-    </row>
-    <row r="41" ht="17" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A41" s="47" t="s">
-        <v>158</v>
-      </c>
-      <c r="B41" s="47"/>
-      <c r="C41" s="47"/>
-      <c r="D41" s="48">
-        <v>0</v>
-      </c>
-      <c r="E41" s="48"/>
-      <c r="F41" s="48"/>
-      <c r="G41" s="48"/>
-      <c r="H41" s="48"/>
-      <c r="I41" s="48"/>
-      <c r="J41" s="48"/>
-      <c r="K41" s="43" t="s">
-        <v>159</v>
-      </c>
-      <c r="L41" s="43"/>
-    </row>
-    <row r="42" ht="17" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A42" s="47" t="s">
-        <v>160</v>
-      </c>
-      <c r="B42" s="47"/>
-      <c r="C42" s="47"/>
-      <c r="D42" s="48">
-        <v>0</v>
-      </c>
-      <c r="E42" s="48"/>
-      <c r="F42" s="48"/>
-      <c r="G42" s="48"/>
-      <c r="H42" s="48"/>
-      <c r="I42" s="48"/>
-      <c r="J42" s="48"/>
-      <c r="K42" s="43" t="s">
-        <v>161</v>
-      </c>
-      <c r="L42" s="43"/>
-    </row>
-    <row r="43" ht="17" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A43" s="51" t="s">
+      <c r="E43" s="48"/>
+      <c r="F43" s="48"/>
+      <c r="G43" s="48"/>
+      <c r="H43" s="48"/>
+      <c r="I43" s="48"/>
+      <c r="J43" s="40" t="s">
         <v>162</v>
       </c>
-      <c r="B43" s="51"/>
-      <c r="C43" s="51"/>
-      <c r="D43" s="52">
-        <v>4500000</v>
-      </c>
-      <c r="E43" s="52"/>
-      <c r="F43" s="52"/>
-      <c r="G43" s="52"/>
-      <c r="H43" s="52"/>
-      <c r="I43" s="52"/>
-      <c r="J43" s="52"/>
-      <c r="K43" s="43" t="s">
+    </row>
+    <row r="44" ht="17" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A44" s="41" t="s">
         <v>163</v>
       </c>
-      <c r="L43" s="43"/>
-    </row>
-    <row r="44" ht="17" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A44" s="45" t="s">
+      <c r="B44" s="41"/>
+      <c r="C44" s="41"/>
+      <c r="D44" s="41"/>
+      <c r="E44" s="41"/>
+      <c r="F44" s="41"/>
+      <c r="G44" s="41"/>
+      <c r="H44" s="41"/>
+      <c r="I44" s="41"/>
+      <c r="J44" s="40" t="s">
         <v>164</v>
       </c>
-      <c r="B44" s="45"/>
-      <c r="C44" s="45"/>
-      <c r="D44" s="45"/>
-      <c r="E44" s="45"/>
-      <c r="F44" s="45"/>
-      <c r="G44" s="45"/>
-      <c r="H44" s="45"/>
-      <c r="I44" s="45"/>
-      <c r="J44" s="45"/>
-      <c r="K44" s="43" t="s">
+    </row>
+    <row r="45" ht="17" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A45" s="43" t="s">
         <v>165</v>
       </c>
-      <c r="L44" s="43"/>
-    </row>
-    <row r="45" ht="17" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A45" s="47" t="s">
+      <c r="B45" s="43"/>
+      <c r="C45" s="43"/>
+      <c r="D45" s="44">
+        <v>35000000</v>
+      </c>
+      <c r="E45" s="44"/>
+      <c r="F45" s="44"/>
+      <c r="G45" s="44"/>
+      <c r="H45" s="44"/>
+      <c r="I45" s="44"/>
+      <c r="J45" s="50"/>
+    </row>
+    <row r="46" ht="17" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A46" s="43" t="s">
         <v>166</v>
       </c>
-      <c r="B45" s="47"/>
-      <c r="C45" s="47"/>
-      <c r="D45" s="48">
-        <v>35000000</v>
-      </c>
-      <c r="E45" s="48"/>
-      <c r="F45" s="48"/>
-      <c r="G45" s="48"/>
-      <c r="H45" s="48"/>
-      <c r="I45" s="48"/>
-      <c r="J45" s="48"/>
-      <c r="K45" s="54"/>
-      <c r="L45" s="54"/>
-    </row>
-    <row r="46" ht="17" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A46" s="47" t="s">
+      <c r="B46" s="43"/>
+      <c r="C46" s="43"/>
+      <c r="D46" s="44">
+        <v>25000000</v>
+      </c>
+      <c r="E46" s="44"/>
+      <c r="F46" s="44"/>
+      <c r="G46" s="44"/>
+      <c r="H46" s="44"/>
+      <c r="I46" s="44"/>
+      <c r="J46" s="50"/>
+    </row>
+    <row r="47" ht="17" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A47" s="43" t="s">
         <v>167</v>
       </c>
-      <c r="B46" s="47"/>
-      <c r="C46" s="47"/>
-      <c r="D46" s="48">
-        <v>25000000</v>
-      </c>
-      <c r="E46" s="48"/>
-      <c r="F46" s="48"/>
-      <c r="G46" s="48"/>
-      <c r="H46" s="48"/>
-      <c r="I46" s="48"/>
-      <c r="J46" s="48"/>
-      <c r="K46" s="54"/>
-      <c r="L46" s="54"/>
-    </row>
-    <row r="47" ht="17" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A47" s="47" t="s">
+      <c r="B47" s="43"/>
+      <c r="C47" s="43"/>
+      <c r="D47" s="44">
+        <v>0</v>
+      </c>
+      <c r="E47" s="44"/>
+      <c r="F47" s="44"/>
+      <c r="G47" s="44"/>
+      <c r="H47" s="44"/>
+      <c r="I47" s="44"/>
+      <c r="J47" s="50"/>
+    </row>
+    <row r="48" ht="17" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A48" s="47" t="s">
         <v>168</v>
       </c>
-      <c r="B47" s="47"/>
-      <c r="C47" s="47"/>
-      <c r="D47" s="48">
-        <v>0</v>
-      </c>
-      <c r="E47" s="48"/>
-      <c r="F47" s="48"/>
-      <c r="G47" s="48"/>
-      <c r="H47" s="48"/>
-      <c r="I47" s="48"/>
-      <c r="J47" s="48"/>
-      <c r="K47" s="54"/>
-      <c r="L47" s="54"/>
-    </row>
-    <row r="48" ht="17" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A48" s="51" t="s">
-        <v>169</v>
-      </c>
-      <c r="B48" s="51"/>
-      <c r="C48" s="51"/>
-      <c r="D48" s="52">
+      <c r="B48" s="47"/>
+      <c r="C48" s="47"/>
+      <c r="D48" s="48">
         <v>10000000</v>
       </c>
-      <c r="E48" s="52"/>
-      <c r="F48" s="52"/>
-      <c r="G48" s="52"/>
-      <c r="H48" s="52"/>
-      <c r="I48" s="52"/>
-      <c r="J48" s="52"/>
-      <c r="K48" s="54"/>
-      <c r="L48" s="54"/>
-    </row>
-    <row r="49" ht="2" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A49" s="55"/>
-      <c r="B49" s="55"/>
-      <c r="C49" s="55"/>
-      <c r="D49" s="55"/>
-      <c r="E49" s="55"/>
-      <c r="F49" s="55"/>
-      <c r="G49" s="55"/>
-      <c r="H49" s="55"/>
-      <c r="I49" s="55"/>
-      <c r="J49" s="55"/>
-      <c r="K49" s="55"/>
-      <c r="L49" s="55"/>
+      <c r="E48" s="48"/>
+      <c r="F48" s="48"/>
+      <c r="G48" s="48"/>
+      <c r="H48" s="48"/>
+      <c r="I48" s="48"/>
+      <c r="J48" s="50"/>
+    </row>
+    <row r="49" ht="2" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A49" s="51"/>
+      <c r="B49" s="51"/>
+      <c r="C49" s="51"/>
+      <c r="D49" s="51"/>
+      <c r="E49" s="51"/>
+      <c r="F49" s="51"/>
+      <c r="G49" s="51"/>
+      <c r="H49" s="51"/>
+      <c r="I49" s="51"/>
+      <c r="J49" s="51"/>
     </row>
   </sheetData>
-  <mergeCells count="107">
-    <mergeCell ref="A1:C3"/>
-    <mergeCell ref="D1:I3"/>
-    <mergeCell ref="K1:L3"/>
-    <mergeCell ref="J1:J3"/>
-    <mergeCell ref="A4:C4"/>
-    <mergeCell ref="D4:J4"/>
-    <mergeCell ref="K4:L4"/>
-    <mergeCell ref="A5:L5"/>
-    <mergeCell ref="J6:L6"/>
+  <mergeCells count="64">
+    <mergeCell ref="A1:B3"/>
+    <mergeCell ref="C1:G3"/>
+    <mergeCell ref="I1:J3"/>
+    <mergeCell ref="H1:H3"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="C4:H4"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="A5:J5"/>
+    <mergeCell ref="I6:J6"/>
     <mergeCell ref="A6:A7"/>
-    <mergeCell ref="B7:C7"/>
-    <mergeCell ref="G7:H7"/>
-    <mergeCell ref="I7:L7"/>
-    <mergeCell ref="B8:D8"/>
-    <mergeCell ref="E8:G8"/>
-    <mergeCell ref="H8:L8"/>
-    <mergeCell ref="C9:D9"/>
-    <mergeCell ref="E9:F9"/>
-    <mergeCell ref="G9:H9"/>
-    <mergeCell ref="I9:J9"/>
-    <mergeCell ref="K9:L9"/>
-    <mergeCell ref="K10:L10"/>
-    <mergeCell ref="A10:A26"/>
-    <mergeCell ref="K11:L11"/>
-    <mergeCell ref="K12:L12"/>
-    <mergeCell ref="K13:L13"/>
-    <mergeCell ref="K14:L14"/>
-    <mergeCell ref="K15:L15"/>
-    <mergeCell ref="K16:L16"/>
-    <mergeCell ref="K17:L17"/>
-    <mergeCell ref="K18:L18"/>
-    <mergeCell ref="K19:L19"/>
-    <mergeCell ref="K20:L20"/>
-    <mergeCell ref="K21:L21"/>
-    <mergeCell ref="K22:L22"/>
-    <mergeCell ref="K23:L23"/>
-    <mergeCell ref="K24:L24"/>
-    <mergeCell ref="K25:L25"/>
-    <mergeCell ref="K26:L26"/>
-    <mergeCell ref="B27:C27"/>
-    <mergeCell ref="D27:E27"/>
-    <mergeCell ref="F27:G27"/>
-    <mergeCell ref="H27:I27"/>
-    <mergeCell ref="K27:L27"/>
-    <mergeCell ref="B28:C28"/>
-    <mergeCell ref="D28:E28"/>
-    <mergeCell ref="F28:G28"/>
-    <mergeCell ref="H28:I28"/>
-    <mergeCell ref="K28:L28"/>
-    <mergeCell ref="A29:J29"/>
-    <mergeCell ref="K29:L29"/>
+    <mergeCell ref="I7:J7"/>
+    <mergeCell ref="B8:C8"/>
+    <mergeCell ref="D8:F8"/>
+    <mergeCell ref="G8:I8"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="D9:E9"/>
+    <mergeCell ref="F9:G9"/>
+    <mergeCell ref="H9:I9"/>
+    <mergeCell ref="A27:B27"/>
+    <mergeCell ref="C27:D27"/>
+    <mergeCell ref="E27:F27"/>
+    <mergeCell ref="G27:H27"/>
+    <mergeCell ref="A28:B28"/>
+    <mergeCell ref="C28:D28"/>
+    <mergeCell ref="E28:F28"/>
+    <mergeCell ref="G28:H28"/>
+    <mergeCell ref="A29:I29"/>
     <mergeCell ref="A30:C30"/>
-    <mergeCell ref="D30:J30"/>
-    <mergeCell ref="K30:L30"/>
+    <mergeCell ref="D30:I30"/>
     <mergeCell ref="A31:C31"/>
-    <mergeCell ref="D31:J31"/>
-    <mergeCell ref="K31:L31"/>
+    <mergeCell ref="D31:I31"/>
     <mergeCell ref="A32:C32"/>
-    <mergeCell ref="D32:J32"/>
-    <mergeCell ref="K32:L32"/>
+    <mergeCell ref="D32:I32"/>
     <mergeCell ref="A33:C33"/>
-    <mergeCell ref="D33:J33"/>
-    <mergeCell ref="K33:L33"/>
+    <mergeCell ref="D33:I33"/>
     <mergeCell ref="A34:C34"/>
-    <mergeCell ref="D34:J34"/>
-    <mergeCell ref="K34:L34"/>
-    <mergeCell ref="A35:J35"/>
-    <mergeCell ref="K35:L35"/>
+    <mergeCell ref="D34:I34"/>
+    <mergeCell ref="A35:I35"/>
     <mergeCell ref="A36:C36"/>
-    <mergeCell ref="D36:J36"/>
-    <mergeCell ref="K36:L36"/>
+    <mergeCell ref="D36:I36"/>
     <mergeCell ref="A37:C37"/>
-    <mergeCell ref="D37:J37"/>
-    <mergeCell ref="K37:L37"/>
+    <mergeCell ref="D37:I37"/>
     <mergeCell ref="A38:C38"/>
-    <mergeCell ref="D38:J38"/>
-    <mergeCell ref="K38:L38"/>
+    <mergeCell ref="D38:I38"/>
     <mergeCell ref="A39:C39"/>
-    <mergeCell ref="D39:J39"/>
-    <mergeCell ref="K39:L39"/>
+    <mergeCell ref="D39:I39"/>
     <mergeCell ref="A40:C40"/>
-    <mergeCell ref="D40:J40"/>
-    <mergeCell ref="K40:L40"/>
+    <mergeCell ref="D40:I40"/>
     <mergeCell ref="A41:C41"/>
-    <mergeCell ref="D41:J41"/>
-    <mergeCell ref="K41:L41"/>
+    <mergeCell ref="D41:I41"/>
     <mergeCell ref="A42:C42"/>
-    <mergeCell ref="D42:J42"/>
-    <mergeCell ref="K42:L42"/>
+    <mergeCell ref="D42:I42"/>
     <mergeCell ref="A43:C43"/>
-    <mergeCell ref="D43:J43"/>
-    <mergeCell ref="K43:L43"/>
-    <mergeCell ref="A44:J44"/>
-    <mergeCell ref="K44:L44"/>
+    <mergeCell ref="D43:I43"/>
+    <mergeCell ref="A44:I44"/>
     <mergeCell ref="A45:C45"/>
-    <mergeCell ref="D45:J45"/>
-    <mergeCell ref="K45:L45"/>
+    <mergeCell ref="D45:I45"/>
     <mergeCell ref="A46:C46"/>
-    <mergeCell ref="D46:J46"/>
-    <mergeCell ref="K46:L46"/>
+    <mergeCell ref="D46:I46"/>
     <mergeCell ref="A47:C47"/>
-    <mergeCell ref="D47:J47"/>
-    <mergeCell ref="K47:L47"/>
+    <mergeCell ref="D47:I47"/>
     <mergeCell ref="A48:C48"/>
-    <mergeCell ref="D48:J48"/>
-    <mergeCell ref="K48:L48"/>
-    <mergeCell ref="A49:L49"/>
+    <mergeCell ref="D48:I48"/>
+    <mergeCell ref="A49:J49"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.4" bottom="0.4" header="0" footer="0"/>
   <pageSetup paperSize="9" orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="0"/>

</xml_diff>

<commit_message>
refactor(ui): simplificar lenguaje de formulas e instructivo a terminos claros y profesionales comprensibles para cualquier contribuyente
</commit_message>
<xml_diff>
--- a/Formulario_210_2024_DIAN_Visual.xlsx
+++ b/Formulario_210_2024_DIAN_Visual.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30326"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="7" documentId="11_18CEEC6B3605EE4023CEDD643B09E4ABB25E49CD" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{67AA0CF1-CBAD-4F57-8841-CF829E1A5056}"/>
+  <xr:revisionPtr revIDLastSave="8" documentId="11_18CEEC6B3605EE4023CEDD643B09E4ABB25E49CD" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{756CD11F-1493-426E-9F4A-6B7D80FC68A0}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3804,7 +3804,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="35" x14ac:knownFonts="1">
+  <fonts count="36" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -4007,6 +4007,11 @@
       <color rgb="FF000000"/>
       <name val="Courier New"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+    </font>
   </fonts>
   <fills count="15">
     <fill>
@@ -4348,7 +4353,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="73">
+  <cellXfs count="74">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -4399,6 +4404,149 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -4411,154 +4559,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="35" fillId="10" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -4575,6 +4583,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -4916,55 +4928,55 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="67" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="18"/>
-      <c r="C1" s="18"/>
-      <c r="D1" s="19" t="s">
+      <c r="B1" s="67"/>
+      <c r="C1" s="67"/>
+      <c r="D1" s="68" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="19"/>
-      <c r="F1" s="19"/>
-      <c r="G1" s="19"/>
-      <c r="H1" s="19"/>
-      <c r="I1" s="20" t="s">
+      <c r="E1" s="68"/>
+      <c r="F1" s="68"/>
+      <c r="G1" s="68"/>
+      <c r="H1" s="68"/>
+      <c r="I1" s="69" t="s">
         <v>2</v>
       </c>
-      <c r="J1" s="20"/>
+      <c r="J1" s="69"/>
     </row>
     <row r="2" spans="1:10" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="18"/>
-      <c r="B2" s="18"/>
-      <c r="C2" s="18"/>
-      <c r="D2" s="19"/>
-      <c r="E2" s="19"/>
-      <c r="F2" s="19"/>
-      <c r="G2" s="19"/>
-      <c r="H2" s="19"/>
-      <c r="I2" s="20"/>
-      <c r="J2" s="20"/>
+      <c r="A2" s="67"/>
+      <c r="B2" s="67"/>
+      <c r="C2" s="67"/>
+      <c r="D2" s="68"/>
+      <c r="E2" s="68"/>
+      <c r="F2" s="68"/>
+      <c r="G2" s="68"/>
+      <c r="H2" s="68"/>
+      <c r="I2" s="69"/>
+      <c r="J2" s="69"/>
     </row>
     <row r="3" spans="1:10" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="18"/>
-      <c r="B3" s="18"/>
-      <c r="C3" s="18"/>
-      <c r="D3" s="19"/>
-      <c r="E3" s="19"/>
-      <c r="F3" s="19"/>
-      <c r="G3" s="19"/>
-      <c r="H3" s="19"/>
-      <c r="I3" s="20"/>
-      <c r="J3" s="20"/>
+      <c r="A3" s="67"/>
+      <c r="B3" s="67"/>
+      <c r="C3" s="67"/>
+      <c r="D3" s="68"/>
+      <c r="E3" s="68"/>
+      <c r="F3" s="68"/>
+      <c r="G3" s="68"/>
+      <c r="H3" s="68"/>
+      <c r="I3" s="69"/>
+      <c r="J3" s="69"/>
     </row>
     <row r="4" spans="1:10" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="22" t="s">
+      <c r="A4" s="34" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="21" t="s">
+      <c r="B4" s="70" t="s">
         <v>4</v>
       </c>
-      <c r="C4" s="21"/>
+      <c r="C4" s="70"/>
       <c r="D4" s="2" t="s">
         <v>5</v>
       </c>
@@ -4974,10 +4986,10 @@
       <c r="F4" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="G4" s="21" t="s">
+      <c r="G4" s="70" t="s">
         <v>8</v>
       </c>
-      <c r="H4" s="21"/>
+      <c r="H4" s="70"/>
       <c r="I4" s="1" t="s">
         <v>9</v>
       </c>
@@ -4986,707 +4998,707 @@
       </c>
     </row>
     <row r="5" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="22"/>
-      <c r="B5" s="23" t="s">
+      <c r="A5" s="34"/>
+      <c r="B5" s="71" t="s">
         <v>11</v>
       </c>
-      <c r="C5" s="23"/>
+      <c r="C5" s="71"/>
       <c r="D5" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="E5" s="23" t="s">
+      <c r="E5" s="71" t="s">
         <v>13</v>
       </c>
-      <c r="F5" s="23"/>
+      <c r="F5" s="71"/>
       <c r="G5" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="H5" s="24" t="s">
+      <c r="H5" s="72" t="s">
         <v>15</v>
       </c>
-      <c r="I5" s="24"/>
+      <c r="I5" s="72"/>
       <c r="J5" s="5" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="6" spans="1:10" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="25" t="s">
+      <c r="A6" s="60" t="s">
         <v>17</v>
       </c>
-      <c r="B6" s="25"/>
-      <c r="C6" s="26" t="s">
+      <c r="B6" s="60"/>
+      <c r="C6" s="61" t="s">
         <v>18</v>
       </c>
-      <c r="D6" s="26"/>
-      <c r="E6" s="26" t="s">
+      <c r="D6" s="61"/>
+      <c r="E6" s="61" t="s">
         <v>19</v>
       </c>
-      <c r="F6" s="26"/>
-      <c r="G6" s="27" t="s">
+      <c r="F6" s="61"/>
+      <c r="G6" s="62" t="s">
         <v>20</v>
       </c>
-      <c r="H6" s="27"/>
-      <c r="I6" s="27"/>
-      <c r="J6" s="27"/>
+      <c r="H6" s="62"/>
+      <c r="I6" s="62"/>
+      <c r="J6" s="62"/>
     </row>
     <row r="7" spans="1:10" ht="26.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="31" t="s">
+      <c r="A7" s="49" t="s">
         <v>21</v>
       </c>
       <c r="B7" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="C7" s="28" t="s">
+      <c r="C7" s="63" t="s">
         <v>23</v>
       </c>
-      <c r="D7" s="28"/>
-      <c r="E7" s="29" t="s">
+      <c r="D7" s="63"/>
+      <c r="E7" s="64" t="s">
         <v>24</v>
       </c>
-      <c r="F7" s="29"/>
-      <c r="G7" s="28" t="s">
+      <c r="F7" s="64"/>
+      <c r="G7" s="63" t="s">
         <v>25</v>
       </c>
-      <c r="H7" s="28"/>
-      <c r="I7" s="30" t="s">
+      <c r="H7" s="63"/>
+      <c r="I7" s="65" t="s">
         <v>26</v>
       </c>
-      <c r="J7" s="30"/>
+      <c r="J7" s="65"/>
     </row>
     <row r="8" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="31"/>
+      <c r="A8" s="49"/>
       <c r="B8" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="C8" s="32" t="s">
+      <c r="C8" s="51" t="s">
         <v>28</v>
       </c>
-      <c r="D8" s="32"/>
-      <c r="E8" s="32" t="s">
+      <c r="D8" s="51"/>
+      <c r="E8" s="51" t="s">
         <v>29</v>
       </c>
-      <c r="F8" s="32"/>
-      <c r="G8" s="32" t="s">
+      <c r="F8" s="51"/>
+      <c r="G8" s="51" t="s">
         <v>30</v>
       </c>
-      <c r="H8" s="32"/>
-      <c r="I8" s="33" t="s">
+      <c r="H8" s="51"/>
+      <c r="I8" s="38" t="s">
         <v>31</v>
       </c>
-      <c r="J8" s="33"/>
+      <c r="J8" s="38"/>
     </row>
     <row r="9" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="31"/>
+      <c r="A9" s="49"/>
       <c r="B9" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="C9" s="34"/>
-      <c r="D9" s="34"/>
-      <c r="E9" s="34"/>
-      <c r="F9" s="34"/>
-      <c r="G9" s="34"/>
-      <c r="H9" s="34"/>
-      <c r="I9" s="35" t="s">
+      <c r="C9" s="50"/>
+      <c r="D9" s="50"/>
+      <c r="E9" s="50"/>
+      <c r="F9" s="50"/>
+      <c r="G9" s="50"/>
+      <c r="H9" s="50"/>
+      <c r="I9" s="66" t="s">
         <v>33</v>
       </c>
-      <c r="J9" s="35"/>
+      <c r="J9" s="66"/>
     </row>
     <row r="10" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="31"/>
+      <c r="A10" s="49"/>
       <c r="B10" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="C10" s="32" t="s">
+      <c r="C10" s="51" t="s">
         <v>35</v>
       </c>
-      <c r="D10" s="32"/>
-      <c r="E10" s="32" t="s">
+      <c r="D10" s="51"/>
+      <c r="E10" s="51" t="s">
         <v>36</v>
       </c>
-      <c r="F10" s="32"/>
-      <c r="G10" s="32" t="s">
+      <c r="F10" s="51"/>
+      <c r="G10" s="51" t="s">
         <v>37</v>
       </c>
-      <c r="H10" s="32"/>
-      <c r="I10" s="33" t="s">
+      <c r="H10" s="51"/>
+      <c r="I10" s="38" t="s">
         <v>38</v>
       </c>
-      <c r="J10" s="33"/>
+      <c r="J10" s="38"/>
     </row>
     <row r="11" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="31"/>
+      <c r="A11" s="49"/>
       <c r="B11" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="C11" s="34"/>
-      <c r="D11" s="34"/>
-      <c r="E11" s="32" t="s">
+      <c r="C11" s="50"/>
+      <c r="D11" s="50"/>
+      <c r="E11" s="51" t="s">
         <v>40</v>
       </c>
-      <c r="F11" s="32"/>
-      <c r="G11" s="32" t="s">
+      <c r="F11" s="51"/>
+      <c r="G11" s="51" t="s">
         <v>41</v>
       </c>
-      <c r="H11" s="32"/>
-      <c r="I11" s="33" t="s">
+      <c r="H11" s="51"/>
+      <c r="I11" s="38" t="s">
         <v>42</v>
       </c>
-      <c r="J11" s="33"/>
+      <c r="J11" s="38"/>
     </row>
     <row r="12" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="31"/>
+      <c r="A12" s="49"/>
       <c r="B12" s="10" t="s">
         <v>43</v>
       </c>
-      <c r="C12" s="36" t="s">
+      <c r="C12" s="73" t="s">
         <v>44</v>
       </c>
-      <c r="D12" s="36"/>
-      <c r="E12" s="36" t="s">
+      <c r="D12" s="59"/>
+      <c r="E12" s="59" t="s">
         <v>45</v>
       </c>
-      <c r="F12" s="36"/>
-      <c r="G12" s="36" t="s">
+      <c r="F12" s="59"/>
+      <c r="G12" s="59" t="s">
         <v>46</v>
       </c>
-      <c r="H12" s="36"/>
-      <c r="I12" s="37" t="s">
+      <c r="H12" s="59"/>
+      <c r="I12" s="41" t="s">
         <v>47</v>
       </c>
-      <c r="J12" s="37"/>
+      <c r="J12" s="41"/>
     </row>
     <row r="13" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="31"/>
+      <c r="A13" s="49"/>
       <c r="B13" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="C13" s="34"/>
-      <c r="D13" s="34"/>
-      <c r="E13" s="34"/>
-      <c r="F13" s="34"/>
-      <c r="G13" s="32" t="s">
+      <c r="C13" s="50"/>
+      <c r="D13" s="50"/>
+      <c r="E13" s="50"/>
+      <c r="F13" s="50"/>
+      <c r="G13" s="51" t="s">
         <v>49</v>
       </c>
-      <c r="H13" s="32"/>
-      <c r="I13" s="33" t="s">
+      <c r="H13" s="51"/>
+      <c r="I13" s="38" t="s">
         <v>50</v>
       </c>
-      <c r="J13" s="33"/>
+      <c r="J13" s="38"/>
     </row>
     <row r="14" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="31"/>
+      <c r="A14" s="49"/>
       <c r="B14" s="11" t="s">
         <v>51</v>
       </c>
-      <c r="C14" s="32" t="s">
+      <c r="C14" s="51" t="s">
         <v>52</v>
       </c>
-      <c r="D14" s="32"/>
-      <c r="E14" s="32" t="s">
+      <c r="D14" s="51"/>
+      <c r="E14" s="51" t="s">
         <v>53</v>
       </c>
-      <c r="F14" s="32"/>
-      <c r="G14" s="32" t="s">
+      <c r="F14" s="51"/>
+      <c r="G14" s="51" t="s">
         <v>54</v>
       </c>
-      <c r="H14" s="32"/>
-      <c r="I14" s="33" t="s">
+      <c r="H14" s="51"/>
+      <c r="I14" s="38" t="s">
         <v>55</v>
       </c>
-      <c r="J14" s="33"/>
+      <c r="J14" s="38"/>
     </row>
     <row r="15" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="31"/>
+      <c r="A15" s="49"/>
       <c r="B15" s="11" t="s">
         <v>56</v>
       </c>
-      <c r="C15" s="32" t="s">
+      <c r="C15" s="51" t="s">
         <v>57</v>
       </c>
-      <c r="D15" s="32"/>
-      <c r="E15" s="32" t="s">
+      <c r="D15" s="51"/>
+      <c r="E15" s="51" t="s">
         <v>58</v>
       </c>
-      <c r="F15" s="32"/>
-      <c r="G15" s="32" t="s">
+      <c r="F15" s="51"/>
+      <c r="G15" s="51" t="s">
         <v>59</v>
       </c>
-      <c r="H15" s="32"/>
-      <c r="I15" s="33" t="s">
+      <c r="H15" s="51"/>
+      <c r="I15" s="38" t="s">
         <v>60</v>
       </c>
-      <c r="J15" s="33"/>
+      <c r="J15" s="38"/>
     </row>
     <row r="16" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="31"/>
+      <c r="A16" s="49"/>
       <c r="B16" s="12" t="s">
         <v>61</v>
       </c>
-      <c r="C16" s="38" t="s">
+      <c r="C16" s="57" t="s">
         <v>62</v>
       </c>
-      <c r="D16" s="38"/>
-      <c r="E16" s="38" t="s">
+      <c r="D16" s="57"/>
+      <c r="E16" s="57" t="s">
         <v>63</v>
       </c>
-      <c r="F16" s="38"/>
-      <c r="G16" s="38" t="s">
+      <c r="F16" s="57"/>
+      <c r="G16" s="57" t="s">
         <v>64</v>
       </c>
-      <c r="H16" s="38"/>
-      <c r="I16" s="39" t="s">
+      <c r="H16" s="57"/>
+      <c r="I16" s="58" t="s">
         <v>65</v>
       </c>
-      <c r="J16" s="39"/>
+      <c r="J16" s="58"/>
     </row>
     <row r="17" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="31"/>
+      <c r="A17" s="49"/>
       <c r="B17" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="C17" s="32" t="s">
+      <c r="C17" s="51" t="s">
         <v>67</v>
       </c>
-      <c r="D17" s="32"/>
-      <c r="E17" s="32" t="s">
+      <c r="D17" s="51"/>
+      <c r="E17" s="51" t="s">
         <v>68</v>
       </c>
-      <c r="F17" s="32"/>
-      <c r="G17" s="32" t="s">
+      <c r="F17" s="51"/>
+      <c r="G17" s="51" t="s">
         <v>69</v>
       </c>
-      <c r="H17" s="32"/>
-      <c r="I17" s="33" t="s">
+      <c r="H17" s="51"/>
+      <c r="I17" s="38" t="s">
         <v>70</v>
       </c>
-      <c r="J17" s="33"/>
+      <c r="J17" s="38"/>
     </row>
     <row r="18" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="31"/>
+      <c r="A18" s="49"/>
       <c r="B18" s="11" t="s">
         <v>71</v>
       </c>
-      <c r="C18" s="32" t="s">
+      <c r="C18" s="51" t="s">
         <v>72</v>
       </c>
-      <c r="D18" s="32"/>
-      <c r="E18" s="32" t="s">
+      <c r="D18" s="51"/>
+      <c r="E18" s="51" t="s">
         <v>73</v>
       </c>
-      <c r="F18" s="32"/>
-      <c r="G18" s="32" t="s">
+      <c r="F18" s="51"/>
+      <c r="G18" s="51" t="s">
         <v>74</v>
       </c>
-      <c r="H18" s="32"/>
-      <c r="I18" s="33" t="s">
+      <c r="H18" s="51"/>
+      <c r="I18" s="38" t="s">
         <v>75</v>
       </c>
-      <c r="J18" s="33"/>
+      <c r="J18" s="38"/>
     </row>
     <row r="19" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="31"/>
+      <c r="A19" s="49"/>
       <c r="B19" s="12" t="s">
         <v>76</v>
       </c>
-      <c r="C19" s="38" t="s">
+      <c r="C19" s="57" t="s">
         <v>77</v>
       </c>
-      <c r="D19" s="38"/>
-      <c r="E19" s="38" t="s">
+      <c r="D19" s="57"/>
+      <c r="E19" s="57" t="s">
         <v>78</v>
       </c>
-      <c r="F19" s="38"/>
-      <c r="G19" s="38" t="s">
+      <c r="F19" s="57"/>
+      <c r="G19" s="57" t="s">
         <v>79</v>
       </c>
-      <c r="H19" s="38"/>
-      <c r="I19" s="39" t="s">
+      <c r="H19" s="57"/>
+      <c r="I19" s="58" t="s">
         <v>80</v>
       </c>
-      <c r="J19" s="39"/>
+      <c r="J19" s="58"/>
     </row>
     <row r="20" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="31"/>
+      <c r="A20" s="49"/>
       <c r="B20" s="13" t="s">
         <v>81</v>
       </c>
-      <c r="C20" s="40" t="s">
+      <c r="C20" s="55" t="s">
         <v>82</v>
       </c>
-      <c r="D20" s="40"/>
-      <c r="E20" s="40" t="s">
+      <c r="D20" s="55"/>
+      <c r="E20" s="55" t="s">
         <v>83</v>
       </c>
-      <c r="F20" s="40"/>
-      <c r="G20" s="40" t="s">
+      <c r="F20" s="55"/>
+      <c r="G20" s="55" t="s">
         <v>84</v>
       </c>
-      <c r="H20" s="40"/>
-      <c r="I20" s="41" t="s">
+      <c r="H20" s="55"/>
+      <c r="I20" s="56" t="s">
         <v>85</v>
       </c>
-      <c r="J20" s="41"/>
+      <c r="J20" s="56"/>
     </row>
     <row r="21" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="31"/>
+      <c r="A21" s="49"/>
       <c r="B21" s="7" t="s">
         <v>86</v>
       </c>
-      <c r="C21" s="34"/>
-      <c r="D21" s="34"/>
-      <c r="E21" s="32" t="s">
+      <c r="C21" s="50"/>
+      <c r="D21" s="50"/>
+      <c r="E21" s="51" t="s">
         <v>87</v>
       </c>
-      <c r="F21" s="32"/>
-      <c r="G21" s="32" t="s">
+      <c r="F21" s="51"/>
+      <c r="G21" s="51" t="s">
         <v>88</v>
       </c>
-      <c r="H21" s="32"/>
-      <c r="I21" s="33" t="s">
+      <c r="H21" s="51"/>
+      <c r="I21" s="38" t="s">
         <v>89</v>
       </c>
-      <c r="J21" s="33"/>
+      <c r="J21" s="38"/>
     </row>
     <row r="22" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="31"/>
+      <c r="A22" s="49"/>
       <c r="B22" s="7" t="s">
         <v>90</v>
       </c>
-      <c r="C22" s="34"/>
-      <c r="D22" s="34"/>
-      <c r="E22" s="32" t="s">
+      <c r="C22" s="50"/>
+      <c r="D22" s="50"/>
+      <c r="E22" s="51" t="s">
         <v>91</v>
       </c>
-      <c r="F22" s="32"/>
-      <c r="G22" s="32" t="s">
+      <c r="F22" s="51"/>
+      <c r="G22" s="51" t="s">
         <v>92</v>
       </c>
-      <c r="H22" s="32"/>
-      <c r="I22" s="33" t="s">
+      <c r="H22" s="51"/>
+      <c r="I22" s="38" t="s">
         <v>93</v>
       </c>
-      <c r="J22" s="33"/>
+      <c r="J22" s="38"/>
     </row>
     <row r="23" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="31"/>
+      <c r="A23" s="49"/>
       <c r="B23" s="7" t="s">
         <v>94</v>
       </c>
-      <c r="C23" s="34"/>
-      <c r="D23" s="34"/>
-      <c r="E23" s="32" t="s">
+      <c r="C23" s="50"/>
+      <c r="D23" s="50"/>
+      <c r="E23" s="51" t="s">
         <v>95</v>
       </c>
-      <c r="F23" s="32"/>
-      <c r="G23" s="32" t="s">
+      <c r="F23" s="51"/>
+      <c r="G23" s="51" t="s">
         <v>96</v>
       </c>
-      <c r="H23" s="32"/>
-      <c r="I23" s="33" t="s">
+      <c r="H23" s="51"/>
+      <c r="I23" s="38" t="s">
         <v>97</v>
       </c>
-      <c r="J23" s="33"/>
+      <c r="J23" s="38"/>
     </row>
     <row r="24" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="31"/>
+      <c r="A24" s="49"/>
       <c r="B24" s="14" t="s">
         <v>98</v>
       </c>
-      <c r="C24" s="42" t="s">
+      <c r="C24" s="36" t="s">
         <v>99</v>
       </c>
-      <c r="D24" s="42"/>
-      <c r="E24" s="42" t="s">
+      <c r="D24" s="36"/>
+      <c r="E24" s="36" t="s">
         <v>100</v>
       </c>
-      <c r="F24" s="42"/>
-      <c r="G24" s="42" t="s">
+      <c r="F24" s="36"/>
+      <c r="G24" s="36" t="s">
         <v>101</v>
       </c>
-      <c r="H24" s="42"/>
+      <c r="H24" s="36"/>
       <c r="I24" s="43" t="s">
         <v>102</v>
       </c>
       <c r="J24" s="43"/>
     </row>
     <row r="25" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="44" t="s">
+      <c r="A25" s="52" t="s">
         <v>103</v>
       </c>
-      <c r="B25" s="44"/>
-      <c r="C25" s="45" t="s">
+      <c r="B25" s="52"/>
+      <c r="C25" s="53" t="s">
         <v>104</v>
       </c>
-      <c r="D25" s="45"/>
-      <c r="E25" s="45" t="s">
+      <c r="D25" s="53"/>
+      <c r="E25" s="53" t="s">
         <v>105</v>
       </c>
-      <c r="F25" s="45"/>
-      <c r="G25" s="45"/>
-      <c r="H25" s="46" t="s">
+      <c r="F25" s="53"/>
+      <c r="G25" s="53"/>
+      <c r="H25" s="54" t="s">
         <v>106</v>
       </c>
-      <c r="I25" s="46"/>
-      <c r="J25" s="46"/>
+      <c r="I25" s="54"/>
+      <c r="J25" s="54"/>
     </row>
     <row r="26" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="47" t="s">
+      <c r="A26" s="44" t="s">
         <v>107</v>
       </c>
-      <c r="B26" s="47"/>
-      <c r="C26" s="48" t="s">
+      <c r="B26" s="44"/>
+      <c r="C26" s="45" t="s">
         <v>108</v>
       </c>
-      <c r="D26" s="48"/>
-      <c r="E26" s="49" t="s">
+      <c r="D26" s="45"/>
+      <c r="E26" s="46" t="s">
         <v>109</v>
       </c>
-      <c r="F26" s="49"/>
-      <c r="G26" s="49"/>
-      <c r="H26" s="50" t="s">
+      <c r="F26" s="46"/>
+      <c r="G26" s="46"/>
+      <c r="H26" s="47" t="s">
         <v>110</v>
       </c>
-      <c r="I26" s="50"/>
-      <c r="J26" s="50"/>
+      <c r="I26" s="47"/>
+      <c r="J26" s="47"/>
     </row>
     <row r="27" spans="1:10" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="54" t="s">
+      <c r="A27" s="48" t="s">
         <v>111</v>
       </c>
-      <c r="B27" s="51" t="s">
+      <c r="B27" s="31" t="s">
         <v>112</v>
       </c>
-      <c r="C27" s="51"/>
-      <c r="D27" s="51"/>
-      <c r="E27" s="52" t="s">
+      <c r="C27" s="31"/>
+      <c r="D27" s="31"/>
+      <c r="E27" s="32" t="s">
         <v>113</v>
       </c>
-      <c r="F27" s="52"/>
-      <c r="G27" s="31" t="s">
+      <c r="F27" s="32"/>
+      <c r="G27" s="49" t="s">
         <v>114</v>
       </c>
       <c r="H27" s="15" t="s">
         <v>115</v>
       </c>
-      <c r="I27" s="53" t="s">
+      <c r="I27" s="33" t="s">
         <v>116</v>
       </c>
-      <c r="J27" s="53"/>
+      <c r="J27" s="33"/>
     </row>
     <row r="28" spans="1:10" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="54"/>
-      <c r="B28" s="51" t="s">
+      <c r="A28" s="48"/>
+      <c r="B28" s="31" t="s">
         <v>34</v>
       </c>
-      <c r="C28" s="51"/>
-      <c r="D28" s="51"/>
-      <c r="E28" s="52" t="s">
+      <c r="C28" s="31"/>
+      <c r="D28" s="31"/>
+      <c r="E28" s="32" t="s">
         <v>117</v>
       </c>
-      <c r="F28" s="52"/>
-      <c r="G28" s="31"/>
+      <c r="F28" s="32"/>
+      <c r="G28" s="49"/>
       <c r="H28" s="15" t="s">
         <v>118</v>
       </c>
-      <c r="I28" s="53" t="s">
+      <c r="I28" s="33" t="s">
         <v>119</v>
       </c>
-      <c r="J28" s="53"/>
+      <c r="J28" s="33"/>
     </row>
     <row r="29" spans="1:10" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="54"/>
-      <c r="B29" s="55" t="s">
+      <c r="A29" s="48"/>
+      <c r="B29" s="39" t="s">
         <v>43</v>
       </c>
-      <c r="C29" s="55"/>
-      <c r="D29" s="55"/>
-      <c r="E29" s="56" t="s">
+      <c r="C29" s="39"/>
+      <c r="D29" s="39"/>
+      <c r="E29" s="40" t="s">
         <v>120</v>
       </c>
-      <c r="F29" s="56"/>
-      <c r="G29" s="31"/>
+      <c r="F29" s="40"/>
+      <c r="G29" s="49"/>
       <c r="H29" s="15" t="s">
         <v>121</v>
       </c>
-      <c r="I29" s="53" t="s">
+      <c r="I29" s="33" t="s">
         <v>122</v>
       </c>
-      <c r="J29" s="53"/>
+      <c r="J29" s="33"/>
     </row>
     <row r="30" spans="1:10" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="54"/>
-      <c r="B30" s="51" t="s">
+      <c r="A30" s="48"/>
+      <c r="B30" s="31" t="s">
         <v>123</v>
       </c>
-      <c r="C30" s="51"/>
-      <c r="D30" s="51"/>
-      <c r="E30" s="52" t="s">
+      <c r="C30" s="31"/>
+      <c r="D30" s="31"/>
+      <c r="E30" s="32" t="s">
         <v>124</v>
       </c>
-      <c r="F30" s="52"/>
-      <c r="G30" s="31"/>
+      <c r="F30" s="32"/>
+      <c r="G30" s="49"/>
       <c r="H30" s="15" t="s">
         <v>125</v>
       </c>
-      <c r="I30" s="53" t="s">
+      <c r="I30" s="33" t="s">
         <v>126</v>
       </c>
-      <c r="J30" s="53"/>
+      <c r="J30" s="33"/>
     </row>
     <row r="31" spans="1:10" ht="18" x14ac:dyDescent="0.25">
-      <c r="A31" s="54"/>
-      <c r="B31" s="57" t="s">
+      <c r="A31" s="48"/>
+      <c r="B31" s="35" t="s">
         <v>127</v>
       </c>
-      <c r="C31" s="57"/>
-      <c r="D31" s="57"/>
-      <c r="E31" s="42" t="s">
+      <c r="C31" s="35"/>
+      <c r="D31" s="35"/>
+      <c r="E31" s="36" t="s">
         <v>128</v>
       </c>
-      <c r="F31" s="42"/>
-      <c r="G31" s="31"/>
+      <c r="F31" s="36"/>
+      <c r="G31" s="49"/>
       <c r="H31" s="15" t="s">
         <v>129</v>
       </c>
-      <c r="I31" s="53" t="s">
+      <c r="I31" s="33" t="s">
         <v>130</v>
       </c>
-      <c r="J31" s="53"/>
+      <c r="J31" s="33"/>
     </row>
     <row r="32" spans="1:10" ht="19.5" x14ac:dyDescent="0.25">
-      <c r="A32" s="22" t="s">
+      <c r="A32" s="34" t="s">
         <v>131</v>
       </c>
-      <c r="B32" s="51" t="s">
+      <c r="B32" s="31" t="s">
         <v>132</v>
       </c>
-      <c r="C32" s="51"/>
-      <c r="D32" s="51"/>
-      <c r="E32" s="52" t="s">
+      <c r="C32" s="31"/>
+      <c r="D32" s="31"/>
+      <c r="E32" s="32" t="s">
         <v>133</v>
       </c>
-      <c r="F32" s="52"/>
-      <c r="G32" s="31"/>
+      <c r="F32" s="32"/>
+      <c r="G32" s="49"/>
       <c r="H32" s="10" t="s">
         <v>134</v>
       </c>
-      <c r="I32" s="37" t="s">
+      <c r="I32" s="41" t="s">
         <v>135</v>
       </c>
-      <c r="J32" s="37"/>
+      <c r="J32" s="41"/>
     </row>
     <row r="33" spans="1:10" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="22"/>
-      <c r="B33" s="51" t="s">
+      <c r="A33" s="34"/>
+      <c r="B33" s="31" t="s">
         <v>34</v>
       </c>
-      <c r="C33" s="51"/>
-      <c r="D33" s="51"/>
-      <c r="E33" s="52" t="s">
+      <c r="C33" s="31"/>
+      <c r="D33" s="31"/>
+      <c r="E33" s="32" t="s">
         <v>136</v>
       </c>
-      <c r="F33" s="52"/>
-      <c r="G33" s="31"/>
+      <c r="F33" s="32"/>
+      <c r="G33" s="49"/>
       <c r="H33" s="8" t="s">
         <v>137</v>
       </c>
-      <c r="I33" s="33" t="s">
+      <c r="I33" s="38" t="s">
         <v>138</v>
       </c>
-      <c r="J33" s="33"/>
+      <c r="J33" s="38"/>
     </row>
     <row r="34" spans="1:10" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="22"/>
-      <c r="B34" s="55" t="s">
+      <c r="A34" s="34"/>
+      <c r="B34" s="39" t="s">
         <v>139</v>
       </c>
-      <c r="C34" s="55"/>
-      <c r="D34" s="55"/>
-      <c r="E34" s="56" t="s">
+      <c r="C34" s="39"/>
+      <c r="D34" s="39"/>
+      <c r="E34" s="40" t="s">
         <v>140</v>
       </c>
-      <c r="F34" s="56"/>
-      <c r="G34" s="31"/>
+      <c r="F34" s="40"/>
+      <c r="G34" s="49"/>
       <c r="H34" s="8" t="s">
         <v>141</v>
       </c>
-      <c r="I34" s="37" t="s">
+      <c r="I34" s="41" t="s">
         <v>142</v>
       </c>
-      <c r="J34" s="37"/>
+      <c r="J34" s="41"/>
     </row>
     <row r="35" spans="1:10" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="22"/>
-      <c r="B35" s="51" t="s">
+      <c r="A35" s="34"/>
+      <c r="B35" s="31" t="s">
         <v>143</v>
       </c>
-      <c r="C35" s="51"/>
-      <c r="D35" s="51"/>
-      <c r="E35" s="52" t="s">
+      <c r="C35" s="31"/>
+      <c r="D35" s="31"/>
+      <c r="E35" s="32" t="s">
         <v>144</v>
       </c>
-      <c r="F35" s="52"/>
-      <c r="G35" s="31"/>
+      <c r="F35" s="32"/>
+      <c r="G35" s="49"/>
       <c r="H35" s="16" t="s">
         <v>145</v>
       </c>
-      <c r="I35" s="58" t="s">
+      <c r="I35" s="42" t="s">
         <v>146</v>
       </c>
-      <c r="J35" s="58"/>
+      <c r="J35" s="42"/>
     </row>
     <row r="36" spans="1:10" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="22"/>
-      <c r="B36" s="51" t="s">
+      <c r="A36" s="34"/>
+      <c r="B36" s="31" t="s">
         <v>147</v>
       </c>
-      <c r="C36" s="51"/>
-      <c r="D36" s="51"/>
-      <c r="E36" s="52" t="s">
+      <c r="C36" s="31"/>
+      <c r="D36" s="31"/>
+      <c r="E36" s="32" t="s">
         <v>148</v>
       </c>
-      <c r="F36" s="52"/>
-      <c r="G36" s="31"/>
+      <c r="F36" s="32"/>
+      <c r="G36" s="49"/>
       <c r="H36" s="15" t="s">
         <v>149</v>
       </c>
-      <c r="I36" s="53" t="s">
+      <c r="I36" s="33" t="s">
         <v>150</v>
       </c>
-      <c r="J36" s="53"/>
+      <c r="J36" s="33"/>
     </row>
     <row r="37" spans="1:10" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="22"/>
-      <c r="B37" s="51" t="s">
+      <c r="A37" s="34"/>
+      <c r="B37" s="31" t="s">
         <v>151</v>
       </c>
-      <c r="C37" s="51"/>
-      <c r="D37" s="51"/>
-      <c r="E37" s="52" t="s">
+      <c r="C37" s="31"/>
+      <c r="D37" s="31"/>
+      <c r="E37" s="32" t="s">
         <v>152</v>
       </c>
-      <c r="F37" s="52"/>
-      <c r="G37" s="31"/>
+      <c r="F37" s="32"/>
+      <c r="G37" s="49"/>
       <c r="H37" s="15" t="s">
         <v>153</v>
       </c>
-      <c r="I37" s="53" t="s">
+      <c r="I37" s="33" t="s">
         <v>154</v>
       </c>
-      <c r="J37" s="53"/>
+      <c r="J37" s="33"/>
     </row>
     <row r="38" spans="1:10" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="22"/>
-      <c r="B38" s="51" t="s">
+      <c r="A38" s="34"/>
+      <c r="B38" s="31" t="s">
         <v>155</v>
       </c>
-      <c r="C38" s="51"/>
-      <c r="D38" s="51"/>
-      <c r="E38" s="52" t="s">
+      <c r="C38" s="31"/>
+      <c r="D38" s="31"/>
+      <c r="E38" s="32" t="s">
         <v>156</v>
       </c>
-      <c r="F38" s="52"/>
-      <c r="G38" s="31"/>
+      <c r="F38" s="32"/>
+      <c r="G38" s="49"/>
       <c r="H38" s="14" t="s">
         <v>157</v>
       </c>
@@ -5696,227 +5708,269 @@
       <c r="J38" s="43"/>
     </row>
     <row r="39" spans="1:10" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="22"/>
-      <c r="B39" s="57" t="s">
+      <c r="A39" s="34"/>
+      <c r="B39" s="35" t="s">
         <v>159</v>
       </c>
-      <c r="C39" s="57"/>
-      <c r="D39" s="57"/>
-      <c r="E39" s="42" t="s">
+      <c r="C39" s="35"/>
+      <c r="D39" s="35"/>
+      <c r="E39" s="36" t="s">
         <v>160</v>
       </c>
-      <c r="F39" s="42"/>
-      <c r="G39" s="31"/>
+      <c r="F39" s="36"/>
+      <c r="G39" s="49"/>
       <c r="H39" s="15" t="s">
         <v>161</v>
       </c>
-      <c r="I39" s="53" t="s">
+      <c r="I39" s="33" t="s">
         <v>162</v>
       </c>
-      <c r="J39" s="53"/>
+      <c r="J39" s="33"/>
     </row>
     <row r="40" spans="1:10" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="22" t="s">
+      <c r="A40" s="34" t="s">
         <v>163</v>
       </c>
-      <c r="B40" s="51" t="s">
+      <c r="B40" s="31" t="s">
         <v>164</v>
       </c>
-      <c r="C40" s="51"/>
-      <c r="D40" s="51"/>
-      <c r="E40" s="52" t="s">
+      <c r="C40" s="31"/>
+      <c r="D40" s="31"/>
+      <c r="E40" s="32" t="s">
         <v>165</v>
       </c>
-      <c r="F40" s="52"/>
-      <c r="G40" s="31"/>
+      <c r="F40" s="32"/>
+      <c r="G40" s="49"/>
       <c r="H40" s="15" t="s">
         <v>166</v>
       </c>
-      <c r="I40" s="53" t="s">
+      <c r="I40" s="33" t="s">
         <v>167</v>
       </c>
-      <c r="J40" s="53"/>
+      <c r="J40" s="33"/>
     </row>
     <row r="41" spans="1:10" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="22"/>
-      <c r="B41" s="51" t="s">
+      <c r="A41" s="34"/>
+      <c r="B41" s="31" t="s">
         <v>168</v>
       </c>
-      <c r="C41" s="51"/>
-      <c r="D41" s="51"/>
-      <c r="E41" s="52" t="s">
+      <c r="C41" s="31"/>
+      <c r="D41" s="31"/>
+      <c r="E41" s="32" t="s">
         <v>169</v>
       </c>
-      <c r="F41" s="52"/>
-      <c r="G41" s="31"/>
+      <c r="F41" s="32"/>
+      <c r="G41" s="49"/>
       <c r="H41" s="15" t="s">
         <v>170</v>
       </c>
-      <c r="I41" s="53" t="s">
+      <c r="I41" s="33" t="s">
         <v>171</v>
       </c>
-      <c r="J41" s="53"/>
+      <c r="J41" s="33"/>
     </row>
     <row r="42" spans="1:10" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="22"/>
-      <c r="B42" s="51" t="s">
+      <c r="A42" s="34"/>
+      <c r="B42" s="31" t="s">
         <v>172</v>
       </c>
-      <c r="C42" s="51"/>
-      <c r="D42" s="51"/>
-      <c r="E42" s="52" t="s">
+      <c r="C42" s="31"/>
+      <c r="D42" s="31"/>
+      <c r="E42" s="32" t="s">
         <v>173</v>
       </c>
-      <c r="F42" s="52"/>
-      <c r="G42" s="31"/>
+      <c r="F42" s="32"/>
+      <c r="G42" s="49"/>
       <c r="H42" s="15" t="s">
         <v>174</v>
       </c>
-      <c r="I42" s="53" t="s">
+      <c r="I42" s="33" t="s">
         <v>175</v>
       </c>
-      <c r="J42" s="53"/>
+      <c r="J42" s="33"/>
     </row>
     <row r="43" spans="1:10" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="22"/>
-      <c r="B43" s="57" t="s">
+      <c r="A43" s="34"/>
+      <c r="B43" s="35" t="s">
         <v>176</v>
       </c>
-      <c r="C43" s="57"/>
-      <c r="D43" s="57"/>
-      <c r="E43" s="42" t="s">
+      <c r="C43" s="35"/>
+      <c r="D43" s="35"/>
+      <c r="E43" s="36" t="s">
         <v>177</v>
       </c>
-      <c r="F43" s="42"/>
-      <c r="G43" s="31"/>
+      <c r="F43" s="36"/>
+      <c r="G43" s="49"/>
       <c r="H43" s="17"/>
-      <c r="I43" s="59"/>
-      <c r="J43" s="59"/>
+      <c r="I43" s="37"/>
+      <c r="J43" s="37"/>
     </row>
     <row r="44" spans="1:10" ht="15" x14ac:dyDescent="0.25">
-      <c r="A44" s="60" t="s">
+      <c r="A44" s="21" t="s">
         <v>178</v>
       </c>
-      <c r="B44" s="60"/>
-      <c r="C44" s="60"/>
-      <c r="D44" s="61" t="s">
+      <c r="B44" s="21"/>
+      <c r="C44" s="21"/>
+      <c r="D44" s="22" t="s">
         <v>179</v>
       </c>
-      <c r="E44" s="61"/>
-      <c r="F44" s="62" t="s">
+      <c r="E44" s="22"/>
+      <c r="F44" s="23" t="s">
         <v>180</v>
       </c>
-      <c r="G44" s="62"/>
-      <c r="H44" s="63" t="s">
+      <c r="G44" s="23"/>
+      <c r="H44" s="24" t="s">
         <v>181</v>
       </c>
-      <c r="I44" s="63"/>
-      <c r="J44" s="63"/>
+      <c r="I44" s="24"/>
+      <c r="J44" s="24"/>
     </row>
     <row r="45" spans="1:10" ht="15" x14ac:dyDescent="0.25">
-      <c r="A45" s="64" t="s">
+      <c r="A45" s="25" t="s">
         <v>182</v>
       </c>
-      <c r="B45" s="64"/>
-      <c r="C45" s="64"/>
-      <c r="D45" s="65" t="s">
+      <c r="B45" s="25"/>
+      <c r="C45" s="25"/>
+      <c r="D45" s="26" t="s">
         <v>183</v>
       </c>
-      <c r="E45" s="65"/>
-      <c r="F45" s="66" t="s">
+      <c r="E45" s="26"/>
+      <c r="F45" s="27" t="s">
         <v>184</v>
       </c>
-      <c r="G45" s="66"/>
-      <c r="H45" s="67" t="s">
+      <c r="G45" s="27"/>
+      <c r="H45" s="28" t="s">
         <v>185</v>
       </c>
-      <c r="I45" s="67"/>
-      <c r="J45" s="67"/>
+      <c r="I45" s="28"/>
+      <c r="J45" s="28"/>
     </row>
     <row r="46" spans="1:10" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="68" t="s">
+      <c r="A46" s="29" t="s">
         <v>186</v>
       </c>
-      <c r="B46" s="68"/>
-      <c r="C46" s="68"/>
-      <c r="D46" s="68"/>
-      <c r="E46" s="68"/>
-      <c r="F46" s="69" t="s">
+      <c r="B46" s="29"/>
+      <c r="C46" s="29"/>
+      <c r="D46" s="29"/>
+      <c r="E46" s="29"/>
+      <c r="F46" s="30" t="s">
         <v>187</v>
       </c>
-      <c r="G46" s="69"/>
-      <c r="H46" s="69"/>
-      <c r="I46" s="69"/>
-      <c r="J46" s="69"/>
+      <c r="G46" s="30"/>
+      <c r="H46" s="30"/>
+      <c r="I46" s="30"/>
+      <c r="J46" s="30"/>
     </row>
     <row r="47" spans="1:10" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="70" t="s">
+      <c r="A47" s="18" t="s">
         <v>188</v>
       </c>
-      <c r="B47" s="70"/>
-      <c r="C47" s="70"/>
-      <c r="D47" s="70"/>
-      <c r="E47" s="70"/>
-      <c r="F47" s="71" t="s">
+      <c r="B47" s="18"/>
+      <c r="C47" s="18"/>
+      <c r="D47" s="18"/>
+      <c r="E47" s="18"/>
+      <c r="F47" s="19" t="s">
         <v>189</v>
       </c>
-      <c r="G47" s="71"/>
-      <c r="H47" s="71"/>
-      <c r="I47" s="72" t="s">
+      <c r="G47" s="19"/>
+      <c r="H47" s="19"/>
+      <c r="I47" s="20" t="s">
         <v>190</v>
       </c>
-      <c r="J47" s="72"/>
+      <c r="J47" s="20"/>
     </row>
   </sheetData>
   <mergeCells count="162">
-    <mergeCell ref="A47:E47"/>
-    <mergeCell ref="F47:H47"/>
-    <mergeCell ref="I47:J47"/>
-    <mergeCell ref="A44:C44"/>
-    <mergeCell ref="D44:E44"/>
-    <mergeCell ref="F44:G44"/>
-    <mergeCell ref="H44:J44"/>
-    <mergeCell ref="A45:C45"/>
-    <mergeCell ref="D45:E45"/>
-    <mergeCell ref="F45:G45"/>
-    <mergeCell ref="H45:J45"/>
-    <mergeCell ref="A46:E46"/>
-    <mergeCell ref="F46:J46"/>
-    <mergeCell ref="B40:D40"/>
-    <mergeCell ref="E40:F40"/>
-    <mergeCell ref="I40:J40"/>
-    <mergeCell ref="A40:A43"/>
-    <mergeCell ref="B41:D41"/>
-    <mergeCell ref="E41:F41"/>
-    <mergeCell ref="I41:J41"/>
-    <mergeCell ref="B42:D42"/>
-    <mergeCell ref="E42:F42"/>
-    <mergeCell ref="I42:J42"/>
-    <mergeCell ref="B43:D43"/>
-    <mergeCell ref="E43:F43"/>
-    <mergeCell ref="I43:J43"/>
-    <mergeCell ref="A32:A39"/>
-    <mergeCell ref="B33:D33"/>
-    <mergeCell ref="E33:F33"/>
-    <mergeCell ref="I33:J33"/>
-    <mergeCell ref="B34:D34"/>
-    <mergeCell ref="E34:F34"/>
-    <mergeCell ref="I34:J34"/>
-    <mergeCell ref="B35:D35"/>
-    <mergeCell ref="E35:F35"/>
-    <mergeCell ref="I35:J35"/>
-    <mergeCell ref="B36:D36"/>
-    <mergeCell ref="E36:F36"/>
-    <mergeCell ref="I36:J36"/>
-    <mergeCell ref="B37:D37"/>
-    <mergeCell ref="E37:F37"/>
-    <mergeCell ref="I37:J37"/>
-    <mergeCell ref="B38:D38"/>
-    <mergeCell ref="E38:F38"/>
-    <mergeCell ref="I38:J38"/>
-    <mergeCell ref="B39:D39"/>
-    <mergeCell ref="E39:F39"/>
-    <mergeCell ref="I39:J39"/>
+    <mergeCell ref="A1:C3"/>
+    <mergeCell ref="D1:H3"/>
+    <mergeCell ref="I1:J3"/>
+    <mergeCell ref="B4:C4"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="A4:A5"/>
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="E5:F5"/>
+    <mergeCell ref="H5:I5"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="C6:D6"/>
+    <mergeCell ref="E6:F6"/>
+    <mergeCell ref="G6:J6"/>
+    <mergeCell ref="C7:D7"/>
+    <mergeCell ref="E7:F7"/>
+    <mergeCell ref="G7:H7"/>
+    <mergeCell ref="I7:J7"/>
+    <mergeCell ref="A7:A24"/>
+    <mergeCell ref="C8:D8"/>
+    <mergeCell ref="E8:F8"/>
+    <mergeCell ref="G8:H8"/>
+    <mergeCell ref="I8:J8"/>
+    <mergeCell ref="C9:D9"/>
+    <mergeCell ref="E9:F9"/>
+    <mergeCell ref="G9:H9"/>
+    <mergeCell ref="I9:J9"/>
+    <mergeCell ref="C10:D10"/>
+    <mergeCell ref="E10:F10"/>
+    <mergeCell ref="G10:H10"/>
+    <mergeCell ref="I10:J10"/>
+    <mergeCell ref="C11:D11"/>
+    <mergeCell ref="E11:F11"/>
+    <mergeCell ref="G11:H11"/>
+    <mergeCell ref="I11:J11"/>
+    <mergeCell ref="C12:D12"/>
+    <mergeCell ref="E12:F12"/>
+    <mergeCell ref="G12:H12"/>
+    <mergeCell ref="I12:J12"/>
+    <mergeCell ref="C13:D13"/>
+    <mergeCell ref="E13:F13"/>
+    <mergeCell ref="G13:H13"/>
+    <mergeCell ref="I13:J13"/>
+    <mergeCell ref="C14:D14"/>
+    <mergeCell ref="E14:F14"/>
+    <mergeCell ref="G14:H14"/>
+    <mergeCell ref="I14:J14"/>
+    <mergeCell ref="C15:D15"/>
+    <mergeCell ref="E15:F15"/>
+    <mergeCell ref="G15:H15"/>
+    <mergeCell ref="I15:J15"/>
+    <mergeCell ref="C16:D16"/>
+    <mergeCell ref="E16:F16"/>
+    <mergeCell ref="G16:H16"/>
+    <mergeCell ref="I16:J16"/>
+    <mergeCell ref="C17:D17"/>
+    <mergeCell ref="E17:F17"/>
+    <mergeCell ref="G17:H17"/>
+    <mergeCell ref="I17:J17"/>
+    <mergeCell ref="C18:D18"/>
+    <mergeCell ref="E18:F18"/>
+    <mergeCell ref="G18:H18"/>
+    <mergeCell ref="I18:J18"/>
+    <mergeCell ref="C19:D19"/>
+    <mergeCell ref="E19:F19"/>
+    <mergeCell ref="G19:H19"/>
+    <mergeCell ref="I19:J19"/>
+    <mergeCell ref="C20:D20"/>
+    <mergeCell ref="E20:F20"/>
+    <mergeCell ref="G20:H20"/>
+    <mergeCell ref="I20:J20"/>
+    <mergeCell ref="C21:D21"/>
+    <mergeCell ref="E21:F21"/>
+    <mergeCell ref="G21:H21"/>
+    <mergeCell ref="I21:J21"/>
+    <mergeCell ref="C22:D22"/>
+    <mergeCell ref="E22:F22"/>
+    <mergeCell ref="G22:H22"/>
+    <mergeCell ref="I22:J22"/>
+    <mergeCell ref="C23:D23"/>
+    <mergeCell ref="E23:F23"/>
+    <mergeCell ref="G23:H23"/>
+    <mergeCell ref="I23:J23"/>
+    <mergeCell ref="C24:D24"/>
+    <mergeCell ref="E24:F24"/>
+    <mergeCell ref="G24:H24"/>
+    <mergeCell ref="I24:J24"/>
+    <mergeCell ref="A25:B25"/>
+    <mergeCell ref="C25:D25"/>
+    <mergeCell ref="E25:G25"/>
+    <mergeCell ref="H25:J25"/>
     <mergeCell ref="A26:B26"/>
     <mergeCell ref="C26:D26"/>
     <mergeCell ref="E26:G26"/>
@@ -5941,96 +5995,54 @@
     <mergeCell ref="B32:D32"/>
     <mergeCell ref="E32:F32"/>
     <mergeCell ref="I32:J32"/>
-    <mergeCell ref="C23:D23"/>
-    <mergeCell ref="E23:F23"/>
-    <mergeCell ref="G23:H23"/>
-    <mergeCell ref="I23:J23"/>
-    <mergeCell ref="C24:D24"/>
-    <mergeCell ref="E24:F24"/>
-    <mergeCell ref="G24:H24"/>
-    <mergeCell ref="I24:J24"/>
-    <mergeCell ref="A25:B25"/>
-    <mergeCell ref="C25:D25"/>
-    <mergeCell ref="E25:G25"/>
-    <mergeCell ref="H25:J25"/>
-    <mergeCell ref="C20:D20"/>
-    <mergeCell ref="E20:F20"/>
-    <mergeCell ref="G20:H20"/>
-    <mergeCell ref="I20:J20"/>
-    <mergeCell ref="C21:D21"/>
-    <mergeCell ref="E21:F21"/>
-    <mergeCell ref="G21:H21"/>
-    <mergeCell ref="I21:J21"/>
-    <mergeCell ref="C22:D22"/>
-    <mergeCell ref="E22:F22"/>
-    <mergeCell ref="G22:H22"/>
-    <mergeCell ref="I22:J22"/>
-    <mergeCell ref="C17:D17"/>
-    <mergeCell ref="E17:F17"/>
-    <mergeCell ref="G17:H17"/>
-    <mergeCell ref="I17:J17"/>
-    <mergeCell ref="C18:D18"/>
-    <mergeCell ref="E18:F18"/>
-    <mergeCell ref="G18:H18"/>
-    <mergeCell ref="I18:J18"/>
-    <mergeCell ref="C19:D19"/>
-    <mergeCell ref="E19:F19"/>
-    <mergeCell ref="G19:H19"/>
-    <mergeCell ref="I19:J19"/>
-    <mergeCell ref="C14:D14"/>
-    <mergeCell ref="E14:F14"/>
-    <mergeCell ref="G14:H14"/>
-    <mergeCell ref="I14:J14"/>
-    <mergeCell ref="C15:D15"/>
-    <mergeCell ref="E15:F15"/>
-    <mergeCell ref="G15:H15"/>
-    <mergeCell ref="I15:J15"/>
-    <mergeCell ref="C16:D16"/>
-    <mergeCell ref="E16:F16"/>
-    <mergeCell ref="G16:H16"/>
-    <mergeCell ref="I16:J16"/>
-    <mergeCell ref="I11:J11"/>
-    <mergeCell ref="C12:D12"/>
-    <mergeCell ref="E12:F12"/>
-    <mergeCell ref="G12:H12"/>
-    <mergeCell ref="I12:J12"/>
-    <mergeCell ref="C13:D13"/>
-    <mergeCell ref="E13:F13"/>
-    <mergeCell ref="G13:H13"/>
-    <mergeCell ref="I13:J13"/>
-    <mergeCell ref="A6:B6"/>
-    <mergeCell ref="C6:D6"/>
-    <mergeCell ref="E6:F6"/>
-    <mergeCell ref="G6:J6"/>
-    <mergeCell ref="C7:D7"/>
-    <mergeCell ref="E7:F7"/>
-    <mergeCell ref="G7:H7"/>
-    <mergeCell ref="I7:J7"/>
-    <mergeCell ref="A7:A24"/>
-    <mergeCell ref="C8:D8"/>
-    <mergeCell ref="E8:F8"/>
-    <mergeCell ref="G8:H8"/>
-    <mergeCell ref="I8:J8"/>
-    <mergeCell ref="C9:D9"/>
-    <mergeCell ref="E9:F9"/>
-    <mergeCell ref="G9:H9"/>
-    <mergeCell ref="I9:J9"/>
-    <mergeCell ref="C10:D10"/>
-    <mergeCell ref="E10:F10"/>
-    <mergeCell ref="G10:H10"/>
-    <mergeCell ref="I10:J10"/>
-    <mergeCell ref="C11:D11"/>
-    <mergeCell ref="E11:F11"/>
-    <mergeCell ref="G11:H11"/>
-    <mergeCell ref="A1:C3"/>
-    <mergeCell ref="D1:H3"/>
-    <mergeCell ref="I1:J3"/>
-    <mergeCell ref="B4:C4"/>
-    <mergeCell ref="G4:H4"/>
-    <mergeCell ref="A4:A5"/>
-    <mergeCell ref="B5:C5"/>
-    <mergeCell ref="E5:F5"/>
-    <mergeCell ref="H5:I5"/>
+    <mergeCell ref="A32:A39"/>
+    <mergeCell ref="B33:D33"/>
+    <mergeCell ref="E33:F33"/>
+    <mergeCell ref="I33:J33"/>
+    <mergeCell ref="B34:D34"/>
+    <mergeCell ref="E34:F34"/>
+    <mergeCell ref="I34:J34"/>
+    <mergeCell ref="B35:D35"/>
+    <mergeCell ref="E35:F35"/>
+    <mergeCell ref="I35:J35"/>
+    <mergeCell ref="B36:D36"/>
+    <mergeCell ref="E36:F36"/>
+    <mergeCell ref="I36:J36"/>
+    <mergeCell ref="B37:D37"/>
+    <mergeCell ref="E37:F37"/>
+    <mergeCell ref="I37:J37"/>
+    <mergeCell ref="B38:D38"/>
+    <mergeCell ref="E38:F38"/>
+    <mergeCell ref="I38:J38"/>
+    <mergeCell ref="B39:D39"/>
+    <mergeCell ref="E39:F39"/>
+    <mergeCell ref="I39:J39"/>
+    <mergeCell ref="B40:D40"/>
+    <mergeCell ref="E40:F40"/>
+    <mergeCell ref="I40:J40"/>
+    <mergeCell ref="A40:A43"/>
+    <mergeCell ref="B41:D41"/>
+    <mergeCell ref="E41:F41"/>
+    <mergeCell ref="I41:J41"/>
+    <mergeCell ref="B42:D42"/>
+    <mergeCell ref="E42:F42"/>
+    <mergeCell ref="I42:J42"/>
+    <mergeCell ref="B43:D43"/>
+    <mergeCell ref="E43:F43"/>
+    <mergeCell ref="I43:J43"/>
+    <mergeCell ref="A47:E47"/>
+    <mergeCell ref="F47:H47"/>
+    <mergeCell ref="I47:J47"/>
+    <mergeCell ref="A44:C44"/>
+    <mergeCell ref="D44:E44"/>
+    <mergeCell ref="F44:G44"/>
+    <mergeCell ref="H44:J44"/>
+    <mergeCell ref="A45:C45"/>
+    <mergeCell ref="D45:E45"/>
+    <mergeCell ref="F45:G45"/>
+    <mergeCell ref="H45:J45"/>
+    <mergeCell ref="A46:E46"/>
+    <mergeCell ref="F46:J46"/>
   </mergeCells>
   <pageMargins left="0.2" right="0.2" top="0.3" bottom="0.3" header="0" footer="0"/>
   <pageSetup paperSize="9" fitToHeight="0" orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295"/>

</xml_diff>